<commit_message>
Size workbook rows from real column widths so long cells stop clipping
Row heights on the three new tables were estimated from raw character counts,
which clipped the longer evidence and correction cells. They are now computed
from the merged block width at the actual font size. The v6.0 sheet-14 height
formula is kept on its own branch so v6.0 stays byte-identical.

Co-authored-by: Mohammad Selim <miles4482@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MIMO_Deployment_v7.0.xlsx
+++ b/MIMO_Deployment_v7.0.xlsx
@@ -658,7 +658,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="301">
+  <cellXfs count="300">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1350,9 +1350,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -12565,7 +12562,7 @@
       </c>
       <c r="O42" s="170" t="n"/>
     </row>
-    <row r="43" ht="40" customHeight="1">
+    <row r="43" ht="42.2" customHeight="1">
       <c r="A43" s="93" t="n">
         <v>1</v>
       </c>
@@ -12628,7 +12625,7 @@
       </c>
       <c r="O43" s="82" t="n"/>
     </row>
-    <row r="44" ht="40" customHeight="1">
+    <row r="44" ht="42.2" customHeight="1">
       <c r="A44" s="97" t="n">
         <v>2</v>
       </c>
@@ -12691,7 +12688,7 @@
       </c>
       <c r="O44" s="82" t="n"/>
     </row>
-    <row r="45" ht="40" customHeight="1">
+    <row r="45" ht="42.2" customHeight="1">
       <c r="A45" s="93" t="n">
         <v>3</v>
       </c>
@@ -12754,7 +12751,7 @@
       </c>
       <c r="O45" s="82" t="n"/>
     </row>
-    <row r="46" ht="40" customHeight="1">
+    <row r="46" ht="42.2" customHeight="1">
       <c r="A46" s="97" t="n">
         <v>4</v>
       </c>
@@ -12817,7 +12814,7 @@
       </c>
       <c r="O46" s="82" t="n"/>
     </row>
-    <row r="47" ht="40" customHeight="1">
+    <row r="47" ht="65" customHeight="1">
       <c r="A47" s="100" t="n">
         <v>5</v>
       </c>
@@ -13071,7 +13068,7 @@
       </c>
       <c r="O54" s="170" t="n"/>
     </row>
-    <row r="55" ht="40" customHeight="1">
+    <row r="55" ht="65" customHeight="1">
       <c r="A55" s="93" t="n">
         <v>1</v>
       </c>
@@ -13134,7 +13131,7 @@
       </c>
       <c r="O55" s="82" t="n"/>
     </row>
-    <row r="56" ht="40" customHeight="1">
+    <row r="56" ht="42.2" customHeight="1">
       <c r="A56" s="97" t="n">
         <v>2</v>
       </c>
@@ -13197,7 +13194,7 @@
       </c>
       <c r="O56" s="82" t="n"/>
     </row>
-    <row r="57" ht="40" customHeight="1">
+    <row r="57" ht="42.2" customHeight="1">
       <c r="A57" s="100" t="n">
         <v>3</v>
       </c>
@@ -13451,7 +13448,7 @@
       </c>
       <c r="O64" s="170" t="n"/>
     </row>
-    <row r="65" ht="40" customHeight="1">
+    <row r="65" ht="30.8" customHeight="1">
       <c r="A65" s="93" t="n">
         <v>1</v>
       </c>
@@ -13514,7 +13511,7 @@
       </c>
       <c r="O65" s="82" t="n"/>
     </row>
-    <row r="66" ht="40" customHeight="1">
+    <row r="66" ht="42.2" customHeight="1">
       <c r="A66" s="97" t="n">
         <v>2</v>
       </c>
@@ -13577,7 +13574,7 @@
       </c>
       <c r="O66" s="82" t="n"/>
     </row>
-    <row r="67" ht="40" customHeight="1">
+    <row r="67" ht="42.2" customHeight="1">
       <c r="A67" s="93" t="n">
         <v>3</v>
       </c>
@@ -13640,7 +13637,7 @@
       </c>
       <c r="O67" s="82" t="n"/>
     </row>
-    <row r="68" ht="40" customHeight="1">
+    <row r="68" ht="42.2" customHeight="1">
       <c r="A68" s="97" t="n">
         <v>4</v>
       </c>
@@ -13703,7 +13700,7 @@
       </c>
       <c r="O68" s="82" t="n"/>
     </row>
-    <row r="69" ht="40" customHeight="1">
+    <row r="69" ht="30.8" customHeight="1">
       <c r="A69" s="100" t="n">
         <v>5</v>
       </c>
@@ -13957,7 +13954,7 @@
       </c>
       <c r="O76" s="170" t="n"/>
     </row>
-    <row r="77" ht="40" customHeight="1">
+    <row r="77" ht="30.8" customHeight="1">
       <c r="A77" s="93" t="n">
         <v>1</v>
       </c>
@@ -14020,7 +14017,7 @@
       </c>
       <c r="O77" s="82" t="n"/>
     </row>
-    <row r="78" ht="40" customHeight="1">
+    <row r="78" ht="30.8" customHeight="1">
       <c r="A78" s="105" t="n">
         <v>2</v>
       </c>
@@ -14274,7 +14271,7 @@
       </c>
       <c r="O85" s="170" t="n"/>
     </row>
-    <row r="86" ht="40" customHeight="1">
+    <row r="86" ht="42.2" customHeight="1">
       <c r="A86" s="93" t="n">
         <v>1</v>
       </c>
@@ -14337,7 +14334,7 @@
       </c>
       <c r="O86" s="82" t="n"/>
     </row>
-    <row r="87" ht="40" customHeight="1">
+    <row r="87" ht="42.2" customHeight="1">
       <c r="A87" s="97" t="n">
         <v>2</v>
       </c>
@@ -14400,7 +14397,7 @@
       </c>
       <c r="O87" s="82" t="n"/>
     </row>
-    <row r="88" ht="40" customHeight="1">
+    <row r="88" ht="30.8" customHeight="1">
       <c r="A88" s="93" t="n">
         <v>3</v>
       </c>
@@ -14463,7 +14460,7 @@
       </c>
       <c r="O88" s="82" t="n"/>
     </row>
-    <row r="89" ht="40" customHeight="1">
+    <row r="89" ht="30.8" customHeight="1">
       <c r="A89" s="105" t="n">
         <v>4</v>
       </c>
@@ -14717,7 +14714,7 @@
       </c>
       <c r="O96" s="170" t="n"/>
     </row>
-    <row r="97" ht="40" customHeight="1">
+    <row r="97" ht="30.8" customHeight="1">
       <c r="A97" s="93" t="n">
         <v>1</v>
       </c>
@@ -14780,7 +14777,7 @@
       </c>
       <c r="O97" s="82" t="n"/>
     </row>
-    <row r="98" ht="40" customHeight="1">
+    <row r="98" ht="42.2" customHeight="1">
       <c r="A98" s="97" t="n">
         <v>2</v>
       </c>
@@ -14843,7 +14840,7 @@
       </c>
       <c r="O98" s="82" t="n"/>
     </row>
-    <row r="99" ht="40" customHeight="1">
+    <row r="99" ht="42.2" customHeight="1">
       <c r="A99" s="100" t="n">
         <v>3</v>
       </c>
@@ -15097,7 +15094,7 @@
       </c>
       <c r="O106" s="170" t="n"/>
     </row>
-    <row r="107" ht="40" customHeight="1">
+    <row r="107" ht="30.8" customHeight="1">
       <c r="A107" s="93" t="n">
         <v>1</v>
       </c>
@@ -15160,7 +15157,7 @@
       </c>
       <c r="O107" s="82" t="n"/>
     </row>
-    <row r="108" ht="40" customHeight="1">
+    <row r="108" ht="30.8" customHeight="1">
       <c r="A108" s="97" t="n">
         <v>2</v>
       </c>
@@ -15223,7 +15220,7 @@
       </c>
       <c r="O108" s="82" t="n"/>
     </row>
-    <row r="109" ht="40" customHeight="1">
+    <row r="109" ht="30.8" customHeight="1">
       <c r="A109" s="93" t="n">
         <v>3</v>
       </c>
@@ -15286,7 +15283,7 @@
       </c>
       <c r="O109" s="82" t="n"/>
     </row>
-    <row r="110" ht="40" customHeight="1">
+    <row r="110" ht="42.2" customHeight="1">
       <c r="A110" s="97" t="n">
         <v>4</v>
       </c>
@@ -15349,7 +15346,7 @@
       </c>
       <c r="O110" s="82" t="n"/>
     </row>
-    <row r="111" ht="40" customHeight="1">
+    <row r="111" ht="42.2" customHeight="1">
       <c r="A111" s="93" t="n">
         <v>5</v>
       </c>
@@ -15412,7 +15409,7 @@
       </c>
       <c r="O111" s="82" t="n"/>
     </row>
-    <row r="112" ht="40" customHeight="1">
+    <row r="112" ht="30.8" customHeight="1">
       <c r="A112" s="97" t="n">
         <v>6</v>
       </c>
@@ -15475,7 +15472,7 @@
       </c>
       <c r="O112" s="82" t="n"/>
     </row>
-    <row r="113" ht="40" customHeight="1">
+    <row r="113" ht="42.2" customHeight="1">
       <c r="A113" s="93" t="n">
         <v>7</v>
       </c>
@@ -15538,7 +15535,7 @@
       </c>
       <c r="O113" s="82" t="n"/>
     </row>
-    <row r="114" ht="40" customHeight="1">
+    <row r="114" ht="30.8" customHeight="1">
       <c r="A114" s="97" t="n">
         <v>8</v>
       </c>
@@ -15601,7 +15598,7 @@
       </c>
       <c r="O114" s="82" t="n"/>
     </row>
-    <row r="115" ht="40" customHeight="1">
+    <row r="115" ht="30.8" customHeight="1">
       <c r="A115" s="93" t="n">
         <v>9</v>
       </c>
@@ -15664,7 +15661,7 @@
       </c>
       <c r="O115" s="82" t="n"/>
     </row>
-    <row r="116" ht="40" customHeight="1">
+    <row r="116" ht="30.8" customHeight="1">
       <c r="A116" s="105" t="n">
         <v>10</v>
       </c>
@@ -15918,7 +15915,7 @@
       </c>
       <c r="O123" s="170" t="n"/>
     </row>
-    <row r="124" ht="40" customHeight="1">
+    <row r="124" ht="42.2" customHeight="1">
       <c r="A124" s="93" t="n">
         <v>1</v>
       </c>
@@ -15981,7 +15978,7 @@
       </c>
       <c r="O124" s="82" t="n"/>
     </row>
-    <row r="125" ht="40" customHeight="1">
+    <row r="125" ht="42.2" customHeight="1">
       <c r="A125" s="97" t="n">
         <v>2</v>
       </c>
@@ -16044,7 +16041,7 @@
       </c>
       <c r="O125" s="82" t="n"/>
     </row>
-    <row r="126" ht="40" customHeight="1">
+    <row r="126" ht="30.8" customHeight="1">
       <c r="A126" s="93" t="n">
         <v>3</v>
       </c>
@@ -16107,7 +16104,7 @@
       </c>
       <c r="O126" s="82" t="n"/>
     </row>
-    <row r="127" ht="40" customHeight="1">
+    <row r="127" ht="30.8" customHeight="1">
       <c r="A127" s="97" t="n">
         <v>4</v>
       </c>
@@ -16170,7 +16167,7 @@
       </c>
       <c r="O127" s="82" t="n"/>
     </row>
-    <row r="128" ht="40" customHeight="1">
+    <row r="128" ht="30.8" customHeight="1">
       <c r="A128" s="93" t="n">
         <v>5</v>
       </c>
@@ -16233,7 +16230,7 @@
       </c>
       <c r="O128" s="82" t="n"/>
     </row>
-    <row r="129" ht="40" customHeight="1">
+    <row r="129" ht="30.8" customHeight="1">
       <c r="A129" s="97" t="n">
         <v>6</v>
       </c>
@@ -16296,7 +16293,7 @@
       </c>
       <c r="O129" s="82" t="n"/>
     </row>
-    <row r="130" ht="40" customHeight="1">
+    <row r="130" ht="30.8" customHeight="1">
       <c r="A130" s="93" t="n">
         <v>7</v>
       </c>
@@ -16359,7 +16356,7 @@
       </c>
       <c r="O130" s="82" t="n"/>
     </row>
-    <row r="131" ht="40" customHeight="1">
+    <row r="131" ht="42.2" customHeight="1">
       <c r="A131" s="97" t="n">
         <v>8</v>
       </c>
@@ -16422,7 +16419,7 @@
       </c>
       <c r="O131" s="82" t="n"/>
     </row>
-    <row r="132" ht="40" customHeight="1">
+    <row r="132" ht="30.8" customHeight="1">
       <c r="A132" s="100" t="n">
         <v>9</v>
       </c>
@@ -16676,7 +16673,7 @@
       </c>
       <c r="O139" s="170" t="n"/>
     </row>
-    <row r="140" ht="40" customHeight="1">
+    <row r="140" ht="42.2" customHeight="1">
       <c r="A140" s="93" t="n">
         <v>1</v>
       </c>
@@ -16739,7 +16736,7 @@
       </c>
       <c r="O140" s="82" t="n"/>
     </row>
-    <row r="141" ht="40" customHeight="1">
+    <row r="141" ht="42.2" customHeight="1">
       <c r="A141" s="97" t="n">
         <v>2</v>
       </c>
@@ -16802,7 +16799,7 @@
       </c>
       <c r="O141" s="82" t="n"/>
     </row>
-    <row r="142" ht="40" customHeight="1">
+    <row r="142" ht="42.2" customHeight="1">
       <c r="A142" s="93" t="n">
         <v>3</v>
       </c>
@@ -16865,7 +16862,7 @@
       </c>
       <c r="O142" s="82" t="n"/>
     </row>
-    <row r="143" ht="40" customHeight="1">
+    <row r="143" ht="30.8" customHeight="1">
       <c r="A143" s="97" t="n">
         <v>4</v>
       </c>
@@ -16928,7 +16925,7 @@
       </c>
       <c r="O143" s="82" t="n"/>
     </row>
-    <row r="144" ht="40" customHeight="1">
+    <row r="144" ht="42.2" customHeight="1">
       <c r="A144" s="93" t="n">
         <v>5</v>
       </c>
@@ -16991,7 +16988,7 @@
       </c>
       <c r="O144" s="82" t="n"/>
     </row>
-    <row r="145" ht="40" customHeight="1">
+    <row r="145" ht="42.2" customHeight="1">
       <c r="A145" s="97" t="n">
         <v>6</v>
       </c>
@@ -17054,7 +17051,7 @@
       </c>
       <c r="O145" s="82" t="n"/>
     </row>
-    <row r="146" ht="40" customHeight="1">
+    <row r="146" ht="30.8" customHeight="1">
       <c r="A146" s="93" t="n">
         <v>7</v>
       </c>
@@ -17117,7 +17114,7 @@
       </c>
       <c r="O146" s="82" t="n"/>
     </row>
-    <row r="147" ht="40" customHeight="1">
+    <row r="147" ht="42.2" customHeight="1">
       <c r="A147" s="97" t="n">
         <v>8</v>
       </c>
@@ -17180,7 +17177,7 @@
       </c>
       <c r="O147" s="82" t="n"/>
     </row>
-    <row r="148" ht="40" customHeight="1">
+    <row r="148" ht="42.2" customHeight="1">
       <c r="A148" s="93" t="n">
         <v>9</v>
       </c>
@@ -17243,7 +17240,7 @@
       </c>
       <c r="O148" s="82" t="n"/>
     </row>
-    <row r="149" ht="40" customHeight="1">
+    <row r="149" ht="42.2" customHeight="1">
       <c r="A149" s="97" t="n">
         <v>10</v>
       </c>
@@ -17306,7 +17303,7 @@
       </c>
       <c r="O149" s="82" t="n"/>
     </row>
-    <row r="150" ht="40" customHeight="1">
+    <row r="150" ht="30.8" customHeight="1">
       <c r="A150" s="93" t="n">
         <v>11</v>
       </c>
@@ -17369,7 +17366,7 @@
       </c>
       <c r="O150" s="82" t="n"/>
     </row>
-    <row r="151" ht="40" customHeight="1">
+    <row r="151" ht="30.8" customHeight="1">
       <c r="A151" s="97" t="n">
         <v>12</v>
       </c>
@@ -17432,7 +17429,7 @@
       </c>
       <c r="O151" s="82" t="n"/>
     </row>
-    <row r="152" ht="40" customHeight="1">
+    <row r="152" ht="30.8" customHeight="1">
       <c r="A152" s="93" t="n">
         <v>13</v>
       </c>
@@ -17495,7 +17492,7 @@
       </c>
       <c r="O152" s="82" t="n"/>
     </row>
-    <row r="153" ht="40" customHeight="1">
+    <row r="153" ht="42.2" customHeight="1">
       <c r="A153" s="105" t="n">
         <v>14</v>
       </c>
@@ -17749,7 +17746,7 @@
       </c>
       <c r="O160" s="170" t="n"/>
     </row>
-    <row r="161" ht="40" customHeight="1">
+    <row r="161" ht="30.8" customHeight="1">
       <c r="A161" s="93" t="n">
         <v>1</v>
       </c>
@@ -17812,7 +17809,7 @@
       </c>
       <c r="O161" s="82" t="n"/>
     </row>
-    <row r="162" ht="40" customHeight="1">
+    <row r="162" ht="42.2" customHeight="1">
       <c r="A162" s="97" t="n">
         <v>2</v>
       </c>
@@ -17875,7 +17872,7 @@
       </c>
       <c r="O162" s="82" t="n"/>
     </row>
-    <row r="163" ht="40" customHeight="1">
+    <row r="163" ht="30.8" customHeight="1">
       <c r="A163" s="93" t="n">
         <v>3</v>
       </c>
@@ -17938,7 +17935,7 @@
       </c>
       <c r="O163" s="82" t="n"/>
     </row>
-    <row r="164" ht="40" customHeight="1">
+    <row r="164" ht="30.8" customHeight="1">
       <c r="A164" s="97" t="n">
         <v>4</v>
       </c>
@@ -18001,7 +17998,7 @@
       </c>
       <c r="O164" s="82" t="n"/>
     </row>
-    <row r="165" ht="40" customHeight="1">
+    <row r="165" ht="42.2" customHeight="1">
       <c r="A165" s="100" t="n">
         <v>5</v>
       </c>
@@ -18255,7 +18252,7 @@
       </c>
       <c r="O172" s="170" t="n"/>
     </row>
-    <row r="173" ht="52" customHeight="1">
+    <row r="173" ht="65" customHeight="1">
       <c r="A173" s="93" t="n">
         <v>1</v>
       </c>
@@ -18318,7 +18315,7 @@
       </c>
       <c r="O173" s="82" t="n"/>
     </row>
-    <row r="174" ht="40" customHeight="1">
+    <row r="174" ht="30.8" customHeight="1">
       <c r="A174" s="97" t="n">
         <v>2</v>
       </c>
@@ -18381,7 +18378,7 @@
       </c>
       <c r="O174" s="82" t="n"/>
     </row>
-    <row r="175" ht="40" customHeight="1">
+    <row r="175" ht="42.2" customHeight="1">
       <c r="A175" s="93" t="n">
         <v>3</v>
       </c>
@@ -18444,7 +18441,7 @@
       </c>
       <c r="O175" s="82" t="n"/>
     </row>
-    <row r="176" ht="40" customHeight="1">
+    <row r="176" ht="30.8" customHeight="1">
       <c r="A176" s="97" t="n">
         <v>4</v>
       </c>
@@ -18507,7 +18504,7 @@
       </c>
       <c r="O176" s="82" t="n"/>
     </row>
-    <row r="177" ht="40" customHeight="1">
+    <row r="177" ht="30.8" customHeight="1">
       <c r="A177" s="93" t="n">
         <v>5</v>
       </c>
@@ -18570,7 +18567,7 @@
       </c>
       <c r="O177" s="82" t="n"/>
     </row>
-    <row r="178" ht="40" customHeight="1">
+    <row r="178" ht="30.8" customHeight="1">
       <c r="A178" s="97" t="n">
         <v>6</v>
       </c>
@@ -18633,7 +18630,7 @@
       </c>
       <c r="O178" s="82" t="n"/>
     </row>
-    <row r="179" ht="40" customHeight="1">
+    <row r="179" ht="30.8" customHeight="1">
       <c r="A179" s="93" t="n">
         <v>7</v>
       </c>
@@ -18696,7 +18693,7 @@
       </c>
       <c r="O179" s="82" t="n"/>
     </row>
-    <row r="180" ht="40" customHeight="1">
+    <row r="180" ht="42.2" customHeight="1">
       <c r="A180" s="105" t="n">
         <v>8</v>
       </c>
@@ -18950,7 +18947,7 @@
       </c>
       <c r="O187" s="170" t="n"/>
     </row>
-    <row r="188" ht="52" customHeight="1">
+    <row r="188" ht="65" customHeight="1">
       <c r="A188" s="93" t="n">
         <v>1</v>
       </c>
@@ -19013,7 +19010,7 @@
       </c>
       <c r="O188" s="82" t="n"/>
     </row>
-    <row r="189" ht="40" customHeight="1">
+    <row r="189" ht="30.8" customHeight="1">
       <c r="A189" s="97" t="n">
         <v>2</v>
       </c>
@@ -19076,7 +19073,7 @@
       </c>
       <c r="O189" s="82" t="n"/>
     </row>
-    <row r="190" ht="40" customHeight="1">
+    <row r="190" ht="53.6" customHeight="1">
       <c r="A190" s="93" t="n">
         <v>3</v>
       </c>
@@ -19139,7 +19136,7 @@
       </c>
       <c r="O190" s="82" t="n"/>
     </row>
-    <row r="191" ht="40" customHeight="1">
+    <row r="191" ht="65" customHeight="1">
       <c r="A191" s="97" t="n">
         <v>4</v>
       </c>
@@ -19202,7 +19199,7 @@
       </c>
       <c r="O191" s="82" t="n"/>
     </row>
-    <row r="192" ht="40" customHeight="1">
+    <row r="192" ht="42.2" customHeight="1">
       <c r="A192" s="93" t="n">
         <v>5</v>
       </c>
@@ -19265,7 +19262,7 @@
       </c>
       <c r="O192" s="82" t="n"/>
     </row>
-    <row r="193" ht="40" customHeight="1">
+    <row r="193" ht="42.2" customHeight="1">
       <c r="A193" s="97" t="n">
         <v>6</v>
       </c>
@@ -19328,7 +19325,7 @@
       </c>
       <c r="O193" s="82" t="n"/>
     </row>
-    <row r="194" ht="40" customHeight="1">
+    <row r="194" ht="42.2" customHeight="1">
       <c r="A194" s="100" t="n">
         <v>7</v>
       </c>
@@ -19582,7 +19579,7 @@
       </c>
       <c r="O201" s="170" t="n"/>
     </row>
-    <row r="202" ht="40" customHeight="1">
+    <row r="202" ht="30.8" customHeight="1">
       <c r="A202" s="93" t="n">
         <v>1</v>
       </c>
@@ -19645,7 +19642,7 @@
       </c>
       <c r="O202" s="82" t="n"/>
     </row>
-    <row r="203" ht="40" customHeight="1">
+    <row r="203" ht="30.8" customHeight="1">
       <c r="A203" s="97" t="n">
         <v>2</v>
       </c>
@@ -19708,7 +19705,7 @@
       </c>
       <c r="O203" s="82" t="n"/>
     </row>
-    <row r="204" ht="40" customHeight="1">
+    <row r="204" ht="30.8" customHeight="1">
       <c r="A204" s="93" t="n">
         <v>3</v>
       </c>
@@ -19771,7 +19768,7 @@
       </c>
       <c r="O204" s="82" t="n"/>
     </row>
-    <row r="205" ht="40" customHeight="1">
+    <row r="205" ht="30.8" customHeight="1">
       <c r="A205" s="97" t="n">
         <v>4</v>
       </c>
@@ -19834,7 +19831,7 @@
       </c>
       <c r="O205" s="82" t="n"/>
     </row>
-    <row r="206" ht="40" customHeight="1">
+    <row r="206" ht="30.8" customHeight="1">
       <c r="A206" s="93" t="n">
         <v>5</v>
       </c>
@@ -19897,7 +19894,7 @@
       </c>
       <c r="O206" s="82" t="n"/>
     </row>
-    <row r="207" ht="40" customHeight="1">
+    <row r="207" ht="30.8" customHeight="1">
       <c r="A207" s="97" t="n">
         <v>6</v>
       </c>
@@ -19960,7 +19957,7 @@
       </c>
       <c r="O207" s="82" t="n"/>
     </row>
-    <row r="208" ht="40" customHeight="1">
+    <row r="208" ht="42.2" customHeight="1">
       <c r="A208" s="93" t="n">
         <v>7</v>
       </c>
@@ -20023,7 +20020,7 @@
       </c>
       <c r="O208" s="82" t="n"/>
     </row>
-    <row r="209" ht="40" customHeight="1">
+    <row r="209" ht="42.2" customHeight="1">
       <c r="A209" s="97" t="n">
         <v>8</v>
       </c>
@@ -20086,7 +20083,7 @@
       </c>
       <c r="O209" s="82" t="n"/>
     </row>
-    <row r="210" ht="40" customHeight="1">
+    <row r="210" ht="30.8" customHeight="1">
       <c r="A210" s="100" t="n">
         <v>9</v>
       </c>
@@ -20340,7 +20337,7 @@
       </c>
       <c r="O217" s="170" t="n"/>
     </row>
-    <row r="218" ht="40" customHeight="1">
+    <row r="218" ht="42.2" customHeight="1">
       <c r="A218" s="93" t="n">
         <v>1</v>
       </c>
@@ -20403,7 +20400,7 @@
       </c>
       <c r="O218" s="82" t="n"/>
     </row>
-    <row r="219" ht="40" customHeight="1">
+    <row r="219" ht="53.6" customHeight="1">
       <c r="A219" s="97" t="n">
         <v>2</v>
       </c>
@@ -20466,7 +20463,7 @@
       </c>
       <c r="O219" s="82" t="n"/>
     </row>
-    <row r="220" ht="40" customHeight="1">
+    <row r="220" ht="30.8" customHeight="1">
       <c r="A220" s="93" t="n">
         <v>3</v>
       </c>
@@ -20529,7 +20526,7 @@
       </c>
       <c r="O220" s="82" t="n"/>
     </row>
-    <row r="221" ht="40" customHeight="1">
+    <row r="221" ht="30.8" customHeight="1">
       <c r="A221" s="97" t="n">
         <v>4</v>
       </c>
@@ -20592,7 +20589,7 @@
       </c>
       <c r="O221" s="82" t="n"/>
     </row>
-    <row r="222" ht="40" customHeight="1">
+    <row r="222" ht="30.8" customHeight="1">
       <c r="A222" s="93" t="n">
         <v>5</v>
       </c>
@@ -20655,7 +20652,7 @@
       </c>
       <c r="O222" s="82" t="n"/>
     </row>
-    <row r="223" ht="40" customHeight="1">
+    <row r="223" ht="30.8" customHeight="1">
       <c r="A223" s="97" t="n">
         <v>6</v>
       </c>
@@ -20718,7 +20715,7 @@
       </c>
       <c r="O223" s="82" t="n"/>
     </row>
-    <row r="224" ht="40" customHeight="1">
+    <row r="224" ht="42.2" customHeight="1">
       <c r="A224" s="93" t="n">
         <v>7</v>
       </c>
@@ -20781,7 +20778,7 @@
       </c>
       <c r="O224" s="82" t="n"/>
     </row>
-    <row r="225" ht="40" customHeight="1">
+    <row r="225" ht="30.8" customHeight="1">
       <c r="A225" s="97" t="n">
         <v>8</v>
       </c>
@@ -20844,7 +20841,7 @@
       </c>
       <c r="O225" s="82" t="n"/>
     </row>
-    <row r="226" ht="40" customHeight="1">
+    <row r="226" ht="42.2" customHeight="1">
       <c r="A226" s="100" t="n">
         <v>9</v>
       </c>
@@ -21098,7 +21095,7 @@
       </c>
       <c r="O233" s="170" t="n"/>
     </row>
-    <row r="234" ht="40" customHeight="1">
+    <row r="234" ht="42.2" customHeight="1">
       <c r="A234" s="93" t="n">
         <v>1</v>
       </c>
@@ -21161,7 +21158,7 @@
       </c>
       <c r="O234" s="82" t="n"/>
     </row>
-    <row r="235" ht="40" customHeight="1">
+    <row r="235" ht="30.8" customHeight="1">
       <c r="A235" s="97" t="n">
         <v>2</v>
       </c>
@@ -21224,7 +21221,7 @@
       </c>
       <c r="O235" s="82" t="n"/>
     </row>
-    <row r="236" ht="40" customHeight="1">
+    <row r="236" ht="30.8" customHeight="1">
       <c r="A236" s="93" t="n">
         <v>3</v>
       </c>
@@ -21287,7 +21284,7 @@
       </c>
       <c r="O236" s="82" t="n"/>
     </row>
-    <row r="237" ht="40" customHeight="1">
+    <row r="237" ht="30.8" customHeight="1">
       <c r="A237" s="97" t="n">
         <v>4</v>
       </c>
@@ -21350,7 +21347,7 @@
       </c>
       <c r="O237" s="82" t="n"/>
     </row>
-    <row r="238" ht="40" customHeight="1">
+    <row r="238" ht="42.2" customHeight="1">
       <c r="A238" s="93" t="n">
         <v>5</v>
       </c>
@@ -21413,7 +21410,7 @@
       </c>
       <c r="O238" s="82" t="n"/>
     </row>
-    <row r="239" ht="40" customHeight="1">
+    <row r="239" ht="42.2" customHeight="1">
       <c r="A239" s="105" t="n">
         <v>6</v>
       </c>
@@ -21667,7 +21664,7 @@
       </c>
       <c r="O246" s="170" t="n"/>
     </row>
-    <row r="247" ht="40" customHeight="1">
+    <row r="247" ht="42.2" customHeight="1">
       <c r="A247" s="93" t="n">
         <v>1</v>
       </c>
@@ -21730,7 +21727,7 @@
       </c>
       <c r="O247" s="82" t="n"/>
     </row>
-    <row r="248" ht="40" customHeight="1">
+    <row r="248" ht="30.8" customHeight="1">
       <c r="A248" s="97" t="n">
         <v>2</v>
       </c>
@@ -21793,7 +21790,7 @@
       </c>
       <c r="O248" s="82" t="n"/>
     </row>
-    <row r="249" ht="40" customHeight="1">
+    <row r="249" ht="53.6" customHeight="1">
       <c r="A249" s="93" t="n">
         <v>3</v>
       </c>
@@ -21856,7 +21853,7 @@
       </c>
       <c r="O249" s="82" t="n"/>
     </row>
-    <row r="250" ht="40" customHeight="1">
+    <row r="250" ht="42.2" customHeight="1">
       <c r="A250" s="97" t="n">
         <v>4</v>
       </c>
@@ -21919,7 +21916,7 @@
       </c>
       <c r="O250" s="82" t="n"/>
     </row>
-    <row r="251" ht="40" customHeight="1">
+    <row r="251" ht="42.2" customHeight="1">
       <c r="A251" s="93" t="n">
         <v>5</v>
       </c>
@@ -21982,7 +21979,7 @@
       </c>
       <c r="O251" s="82" t="n"/>
     </row>
-    <row r="252" ht="40" customHeight="1">
+    <row r="252" ht="42.2" customHeight="1">
       <c r="A252" s="97" t="n">
         <v>6</v>
       </c>
@@ -22045,7 +22042,7 @@
       </c>
       <c r="O252" s="82" t="n"/>
     </row>
-    <row r="253" ht="40" customHeight="1">
+    <row r="253" ht="42.2" customHeight="1">
       <c r="A253" s="93" t="n">
         <v>7</v>
       </c>
@@ -22108,7 +22105,7 @@
       </c>
       <c r="O253" s="82" t="n"/>
     </row>
-    <row r="254" ht="40" customHeight="1">
+    <row r="254" ht="42.2" customHeight="1">
       <c r="A254" s="97" t="n">
         <v>8</v>
       </c>
@@ -22171,7 +22168,7 @@
       </c>
       <c r="O254" s="82" t="n"/>
     </row>
-    <row r="255" ht="40" customHeight="1">
+    <row r="255" ht="42.2" customHeight="1">
       <c r="A255" s="93" t="n">
         <v>9</v>
       </c>
@@ -22234,7 +22231,7 @@
       </c>
       <c r="O255" s="82" t="n"/>
     </row>
-    <row r="256" ht="40" customHeight="1">
+    <row r="256" ht="42.2" customHeight="1">
       <c r="A256" s="97" t="n">
         <v>10</v>
       </c>
@@ -22297,7 +22294,7 @@
       </c>
       <c r="O256" s="82" t="n"/>
     </row>
-    <row r="257" ht="40" customHeight="1">
+    <row r="257" ht="30.8" customHeight="1">
       <c r="A257" s="100" t="n">
         <v>11</v>
       </c>
@@ -22551,7 +22548,7 @@
       </c>
       <c r="O264" s="170" t="n"/>
     </row>
-    <row r="265" ht="40" customHeight="1">
+    <row r="265" ht="30.8" customHeight="1">
       <c r="A265" s="93" t="n">
         <v>1</v>
       </c>
@@ -22614,7 +22611,7 @@
       </c>
       <c r="O265" s="82" t="n"/>
     </row>
-    <row r="266" ht="40" customHeight="1">
+    <row r="266" ht="30.8" customHeight="1">
       <c r="A266" s="97" t="n">
         <v>2</v>
       </c>
@@ -22677,7 +22674,7 @@
       </c>
       <c r="O266" s="82" t="n"/>
     </row>
-    <row r="267" ht="40" customHeight="1">
+    <row r="267" ht="42.2" customHeight="1">
       <c r="A267" s="93" t="n">
         <v>3</v>
       </c>
@@ -22740,7 +22737,7 @@
       </c>
       <c r="O267" s="82" t="n"/>
     </row>
-    <row r="268" ht="40" customHeight="1">
+    <row r="268" ht="42.2" customHeight="1">
       <c r="A268" s="97" t="n">
         <v>4</v>
       </c>
@@ -22803,7 +22800,7 @@
       </c>
       <c r="O268" s="82" t="n"/>
     </row>
-    <row r="269" ht="40" customHeight="1">
+    <row r="269" ht="30.8" customHeight="1">
       <c r="A269" s="93" t="n">
         <v>5</v>
       </c>
@@ -22866,7 +22863,7 @@
       </c>
       <c r="O269" s="82" t="n"/>
     </row>
-    <row r="270" ht="40" customHeight="1">
+    <row r="270" ht="42.2" customHeight="1">
       <c r="A270" s="97" t="n">
         <v>6</v>
       </c>
@@ -22929,7 +22926,7 @@
       </c>
       <c r="O270" s="82" t="n"/>
     </row>
-    <row r="271" ht="40" customHeight="1">
+    <row r="271" ht="30.8" customHeight="1">
       <c r="A271" s="93" t="n">
         <v>7</v>
       </c>
@@ -22992,7 +22989,7 @@
       </c>
       <c r="O271" s="82" t="n"/>
     </row>
-    <row r="272" ht="40" customHeight="1">
+    <row r="272" ht="30.8" customHeight="1">
       <c r="A272" s="97" t="n">
         <v>8</v>
       </c>
@@ -23055,7 +23052,7 @@
       </c>
       <c r="O272" s="82" t="n"/>
     </row>
-    <row r="273" ht="40" customHeight="1">
+    <row r="273" ht="30.8" customHeight="1">
       <c r="A273" s="93" t="n">
         <v>9</v>
       </c>
@@ -23118,7 +23115,7 @@
       </c>
       <c r="O273" s="82" t="n"/>
     </row>
-    <row r="274" ht="40" customHeight="1">
+    <row r="274" ht="30.8" customHeight="1">
       <c r="A274" s="97" t="n">
         <v>10</v>
       </c>
@@ -23181,7 +23178,7 @@
       </c>
       <c r="O274" s="82" t="n"/>
     </row>
-    <row r="275" ht="40" customHeight="1">
+    <row r="275" ht="42.2" customHeight="1">
       <c r="A275" s="100" t="n">
         <v>11</v>
       </c>
@@ -23435,7 +23432,7 @@
       </c>
       <c r="O282" s="170" t="n"/>
     </row>
-    <row r="283" ht="40" customHeight="1">
+    <row r="283" ht="30.8" customHeight="1">
       <c r="A283" s="93" t="n">
         <v>1</v>
       </c>
@@ -23498,7 +23495,7 @@
       </c>
       <c r="O283" s="82" t="n"/>
     </row>
-    <row r="284" ht="40" customHeight="1">
+    <row r="284" ht="30.8" customHeight="1">
       <c r="A284" s="97" t="n">
         <v>2</v>
       </c>
@@ -23561,7 +23558,7 @@
       </c>
       <c r="O284" s="82" t="n"/>
     </row>
-    <row r="285" ht="40" customHeight="1">
+    <row r="285" ht="30.8" customHeight="1">
       <c r="A285" s="93" t="n">
         <v>3</v>
       </c>
@@ -23624,7 +23621,7 @@
       </c>
       <c r="O285" s="82" t="n"/>
     </row>
-    <row r="286" ht="40" customHeight="1">
+    <row r="286" ht="30.8" customHeight="1">
       <c r="A286" s="97" t="n">
         <v>4</v>
       </c>
@@ -23687,7 +23684,7 @@
       </c>
       <c r="O286" s="82" t="n"/>
     </row>
-    <row r="287" ht="40" customHeight="1">
+    <row r="287" ht="30.8" customHeight="1">
       <c r="A287" s="93" t="n">
         <v>5</v>
       </c>
@@ -23750,7 +23747,7 @@
       </c>
       <c r="O287" s="82" t="n"/>
     </row>
-    <row r="288" ht="40" customHeight="1">
+    <row r="288" ht="30.8" customHeight="1">
       <c r="A288" s="105" t="n">
         <v>6</v>
       </c>
@@ -24004,7 +24001,7 @@
       </c>
       <c r="O295" s="170" t="n"/>
     </row>
-    <row r="296" ht="40" customHeight="1">
+    <row r="296" ht="42.2" customHeight="1">
       <c r="A296" s="93" t="n">
         <v>1</v>
       </c>
@@ -24067,7 +24064,7 @@
       </c>
       <c r="O296" s="82" t="n"/>
     </row>
-    <row r="297" ht="40" customHeight="1">
+    <row r="297" ht="30.8" customHeight="1">
       <c r="A297" s="97" t="n">
         <v>2</v>
       </c>
@@ -24130,7 +24127,7 @@
       </c>
       <c r="O297" s="82" t="n"/>
     </row>
-    <row r="298" ht="40" customHeight="1">
+    <row r="298" ht="30.8" customHeight="1">
       <c r="A298" s="93" t="n">
         <v>3</v>
       </c>
@@ -24193,7 +24190,7 @@
       </c>
       <c r="O298" s="82" t="n"/>
     </row>
-    <row r="299" ht="40" customHeight="1">
+    <row r="299" ht="30.8" customHeight="1">
       <c r="A299" s="97" t="n">
         <v>4</v>
       </c>
@@ -24256,7 +24253,7 @@
       </c>
       <c r="O299" s="82" t="n"/>
     </row>
-    <row r="300" ht="40" customHeight="1">
+    <row r="300" ht="30.8" customHeight="1">
       <c r="A300" s="93" t="n">
         <v>5</v>
       </c>
@@ -24319,7 +24316,7 @@
       </c>
       <c r="O300" s="82" t="n"/>
     </row>
-    <row r="301" ht="40" customHeight="1">
+    <row r="301" ht="30.8" customHeight="1">
       <c r="A301" s="97" t="n">
         <v>6</v>
       </c>
@@ -24382,7 +24379,7 @@
       </c>
       <c r="O301" s="82" t="n"/>
     </row>
-    <row r="302" ht="40" customHeight="1">
+    <row r="302" ht="30.8" customHeight="1">
       <c r="A302" s="93" t="n">
         <v>7</v>
       </c>
@@ -24445,7 +24442,7 @@
       </c>
       <c r="O302" s="82" t="n"/>
     </row>
-    <row r="303" ht="40" customHeight="1">
+    <row r="303" ht="30.8" customHeight="1">
       <c r="A303" s="97" t="n">
         <v>8</v>
       </c>
@@ -24508,7 +24505,7 @@
       </c>
       <c r="O303" s="82" t="n"/>
     </row>
-    <row r="304" ht="40" customHeight="1">
+    <row r="304" ht="30.8" customHeight="1">
       <c r="A304" s="93" t="n">
         <v>9</v>
       </c>
@@ -24571,7 +24568,7 @@
       </c>
       <c r="O304" s="82" t="n"/>
     </row>
-    <row r="305" ht="40" customHeight="1">
+    <row r="305" ht="30.8" customHeight="1">
       <c r="A305" s="97" t="n">
         <v>10</v>
       </c>
@@ -24634,7 +24631,7 @@
       </c>
       <c r="O305" s="82" t="n"/>
     </row>
-    <row r="306" ht="40" customHeight="1">
+    <row r="306" ht="30.8" customHeight="1">
       <c r="A306" s="93" t="n">
         <v>11</v>
       </c>
@@ -24697,7 +24694,7 @@
       </c>
       <c r="O306" s="82" t="n"/>
     </row>
-    <row r="307" ht="40" customHeight="1">
+    <row r="307" ht="42.2" customHeight="1">
       <c r="A307" s="97" t="n">
         <v>12</v>
       </c>
@@ -24760,7 +24757,7 @@
       </c>
       <c r="O307" s="82" t="n"/>
     </row>
-    <row r="308" ht="40" customHeight="1">
+    <row r="308" ht="30.8" customHeight="1">
       <c r="A308" s="93" t="n">
         <v>13</v>
       </c>
@@ -24823,7 +24820,7 @@
       </c>
       <c r="O308" s="82" t="n"/>
     </row>
-    <row r="309" ht="40" customHeight="1">
+    <row r="309" ht="30.8" customHeight="1">
       <c r="A309" s="105" t="n">
         <v>14</v>
       </c>
@@ -25077,7 +25074,7 @@
       </c>
       <c r="O316" s="170" t="n"/>
     </row>
-    <row r="317" ht="40" customHeight="1">
+    <row r="317" ht="30.8" customHeight="1">
       <c r="A317" s="93" t="n">
         <v>1</v>
       </c>
@@ -25140,7 +25137,7 @@
       </c>
       <c r="O317" s="82" t="n"/>
     </row>
-    <row r="318" ht="40" customHeight="1">
+    <row r="318" ht="42.2" customHeight="1">
       <c r="A318" s="97" t="n">
         <v>2</v>
       </c>
@@ -25203,7 +25200,7 @@
       </c>
       <c r="O318" s="82" t="n"/>
     </row>
-    <row r="319" ht="40" customHeight="1">
+    <row r="319" ht="30.8" customHeight="1">
       <c r="A319" s="93" t="n">
         <v>3</v>
       </c>
@@ -25266,7 +25263,7 @@
       </c>
       <c r="O319" s="82" t="n"/>
     </row>
-    <row r="320" ht="40" customHeight="1">
+    <row r="320" ht="42.2" customHeight="1">
       <c r="A320" s="97" t="n">
         <v>4</v>
       </c>
@@ -25329,7 +25326,7 @@
       </c>
       <c r="O320" s="82" t="n"/>
     </row>
-    <row r="321" ht="40" customHeight="1">
+    <row r="321" ht="30.8" customHeight="1">
       <c r="A321" s="93" t="n">
         <v>5</v>
       </c>
@@ -25392,7 +25389,7 @@
       </c>
       <c r="O321" s="82" t="n"/>
     </row>
-    <row r="322" ht="40" customHeight="1">
+    <row r="322" ht="30.8" customHeight="1">
       <c r="A322" s="97" t="n">
         <v>6</v>
       </c>
@@ -25455,7 +25452,7 @@
       </c>
       <c r="O322" s="82" t="n"/>
     </row>
-    <row r="323" ht="40" customHeight="1">
+    <row r="323" ht="30.8" customHeight="1">
       <c r="A323" s="93" t="n">
         <v>7</v>
       </c>
@@ -25518,7 +25515,7 @@
       </c>
       <c r="O323" s="82" t="n"/>
     </row>
-    <row r="324" ht="40" customHeight="1">
+    <row r="324" ht="30.8" customHeight="1">
       <c r="A324" s="97" t="n">
         <v>8</v>
       </c>
@@ -25581,7 +25578,7 @@
       </c>
       <c r="O324" s="82" t="n"/>
     </row>
-    <row r="325" ht="40" customHeight="1">
+    <row r="325" ht="42.2" customHeight="1">
       <c r="A325" s="93" t="n">
         <v>9</v>
       </c>
@@ -25644,7 +25641,7 @@
       </c>
       <c r="O325" s="82" t="n"/>
     </row>
-    <row r="326" ht="40" customHeight="1">
+    <row r="326" ht="30.8" customHeight="1">
       <c r="A326" s="105" t="n">
         <v>10</v>
       </c>
@@ -25898,7 +25895,7 @@
       </c>
       <c r="O333" s="170" t="n"/>
     </row>
-    <row r="334" ht="40" customHeight="1">
+    <row r="334" ht="30.8" customHeight="1">
       <c r="A334" s="93" t="n">
         <v>1</v>
       </c>
@@ -25961,7 +25958,7 @@
       </c>
       <c r="O334" s="82" t="n"/>
     </row>
-    <row r="335" ht="40" customHeight="1">
+    <row r="335" ht="30.8" customHeight="1">
       <c r="A335" s="97" t="n">
         <v>2</v>
       </c>
@@ -26024,7 +26021,7 @@
       </c>
       <c r="O335" s="82" t="n"/>
     </row>
-    <row r="336" ht="40" customHeight="1">
+    <row r="336" ht="30.8" customHeight="1">
       <c r="A336" s="93" t="n">
         <v>3</v>
       </c>
@@ -26087,7 +26084,7 @@
       </c>
       <c r="O336" s="82" t="n"/>
     </row>
-    <row r="337" ht="40" customHeight="1">
+    <row r="337" ht="30.8" customHeight="1">
       <c r="A337" s="97" t="n">
         <v>4</v>
       </c>
@@ -26150,7 +26147,7 @@
       </c>
       <c r="O337" s="82" t="n"/>
     </row>
-    <row r="338" ht="40" customHeight="1">
+    <row r="338" ht="30.8" customHeight="1">
       <c r="A338" s="100" t="n">
         <v>5</v>
       </c>
@@ -26404,7 +26401,7 @@
       </c>
       <c r="O345" s="170" t="n"/>
     </row>
-    <row r="346" ht="40" customHeight="1">
+    <row r="346" ht="30.8" customHeight="1">
       <c r="A346" s="93" t="n">
         <v>1</v>
       </c>
@@ -26467,7 +26464,7 @@
       </c>
       <c r="O346" s="82" t="n"/>
     </row>
-    <row r="347" ht="40" customHeight="1">
+    <row r="347" ht="30.8" customHeight="1">
       <c r="A347" s="97" t="n">
         <v>2</v>
       </c>
@@ -26530,7 +26527,7 @@
       </c>
       <c r="O347" s="82" t="n"/>
     </row>
-    <row r="348" ht="40" customHeight="1">
+    <row r="348" ht="30.8" customHeight="1">
       <c r="A348" s="93" t="n">
         <v>3</v>
       </c>
@@ -26593,7 +26590,7 @@
       </c>
       <c r="O348" s="82" t="n"/>
     </row>
-    <row r="349" ht="40" customHeight="1">
+    <row r="349" ht="30.8" customHeight="1">
       <c r="A349" s="97" t="n">
         <v>4</v>
       </c>
@@ -26656,7 +26653,7 @@
       </c>
       <c r="O349" s="82" t="n"/>
     </row>
-    <row r="350" ht="40" customHeight="1">
+    <row r="350" ht="30.8" customHeight="1">
       <c r="A350" s="100" t="n">
         <v>5</v>
       </c>
@@ -26910,7 +26907,7 @@
       </c>
       <c r="O357" s="170" t="n"/>
     </row>
-    <row r="358" ht="40" customHeight="1">
+    <row r="358" ht="42.2" customHeight="1">
       <c r="A358" s="93" t="n">
         <v>1</v>
       </c>
@@ -26973,7 +26970,7 @@
       </c>
       <c r="O358" s="82" t="n"/>
     </row>
-    <row r="359" ht="40" customHeight="1">
+    <row r="359" ht="42.2" customHeight="1">
       <c r="A359" s="97" t="n">
         <v>2</v>
       </c>
@@ -27036,7 +27033,7 @@
       </c>
       <c r="O359" s="82" t="n"/>
     </row>
-    <row r="360" ht="40" customHeight="1">
+    <row r="360" ht="30.8" customHeight="1">
       <c r="A360" s="93" t="n">
         <v>3</v>
       </c>
@@ -27099,7 +27096,7 @@
       </c>
       <c r="O360" s="82" t="n"/>
     </row>
-    <row r="361" ht="40" customHeight="1">
+    <row r="361" ht="30.8" customHeight="1">
       <c r="A361" s="97" t="n">
         <v>4</v>
       </c>
@@ -27162,7 +27159,7 @@
       </c>
       <c r="O361" s="82" t="n"/>
     </row>
-    <row r="362" ht="40" customHeight="1">
+    <row r="362" ht="30.8" customHeight="1">
       <c r="A362" s="93" t="n">
         <v>5</v>
       </c>
@@ -27225,7 +27222,7 @@
       </c>
       <c r="O362" s="82" t="n"/>
     </row>
-    <row r="363" ht="40" customHeight="1">
+    <row r="363" ht="30.8" customHeight="1">
       <c r="A363" s="97" t="n">
         <v>6</v>
       </c>
@@ -27288,7 +27285,7 @@
       </c>
       <c r="O363" s="82" t="n"/>
     </row>
-    <row r="364" ht="40" customHeight="1">
+    <row r="364" ht="30.8" customHeight="1">
       <c r="A364" s="93" t="n">
         <v>7</v>
       </c>
@@ -27351,7 +27348,7 @@
       </c>
       <c r="O364" s="82" t="n"/>
     </row>
-    <row r="365" ht="40" customHeight="1">
+    <row r="365" ht="42.2" customHeight="1">
       <c r="A365" s="105" t="n">
         <v>8</v>
       </c>
@@ -27605,7 +27602,7 @@
       </c>
       <c r="O372" s="170" t="n"/>
     </row>
-    <row r="373" ht="40" customHeight="1">
+    <row r="373" ht="42.2" customHeight="1">
       <c r="A373" s="93" t="n">
         <v>1</v>
       </c>
@@ -27668,7 +27665,7 @@
       </c>
       <c r="O373" s="82" t="n"/>
     </row>
-    <row r="374" ht="40" customHeight="1">
+    <row r="374" ht="42.2" customHeight="1">
       <c r="A374" s="97" t="n">
         <v>2</v>
       </c>
@@ -27731,7 +27728,7 @@
       </c>
       <c r="O374" s="82" t="n"/>
     </row>
-    <row r="375" ht="40" customHeight="1">
+    <row r="375" ht="42.2" customHeight="1">
       <c r="A375" s="100" t="n">
         <v>3</v>
       </c>
@@ -27985,7 +27982,7 @@
       </c>
       <c r="O382" s="170" t="n"/>
     </row>
-    <row r="383" ht="40" customHeight="1">
+    <row r="383" ht="42.2" customHeight="1">
       <c r="A383" s="93" t="n">
         <v>1</v>
       </c>
@@ -28048,7 +28045,7 @@
       </c>
       <c r="O383" s="82" t="n"/>
     </row>
-    <row r="384" ht="40" customHeight="1">
+    <row r="384" ht="42.2" customHeight="1">
       <c r="A384" s="97" t="n">
         <v>2</v>
       </c>
@@ -28111,7 +28108,7 @@
       </c>
       <c r="O384" s="82" t="n"/>
     </row>
-    <row r="385" ht="40" customHeight="1">
+    <row r="385" ht="42.2" customHeight="1">
       <c r="A385" s="93" t="n">
         <v>3</v>
       </c>
@@ -28174,7 +28171,7 @@
       </c>
       <c r="O385" s="82" t="n"/>
     </row>
-    <row r="386" ht="40" customHeight="1">
+    <row r="386" ht="42.2" customHeight="1">
       <c r="A386" s="105" t="n">
         <v>4</v>
       </c>
@@ -45342,16 +45339,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="33" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="41" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -45406,7 +45403,7 @@
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
     </row>
-    <row r="5" ht="176" customHeight="1">
+    <row r="5" ht="153" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>The trial did not fail — it never ran the experiment it was designed to run.
@@ -45518,7 +45515,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="26" customHeight="1">
+    <row r="10" ht="31.8" customHeight="1">
       <c r="A10" s="225" t="n">
         <v>1</v>
       </c>
@@ -45573,7 +45570,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="26" customHeight="1">
+    <row r="11" ht="31.8" customHeight="1">
       <c r="A11" s="231" t="n">
         <v>2</v>
       </c>
@@ -45628,7 +45625,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="26" customHeight="1">
+    <row r="12" ht="31.8" customHeight="1">
       <c r="A12" s="225" t="n">
         <v>3</v>
       </c>
@@ -45683,7 +45680,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1">
+    <row r="13" ht="77.40000000000001" customHeight="1">
       <c r="A13" s="231" t="n">
         <v>4</v>
       </c>
@@ -45738,7 +45735,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="37" customHeight="1">
+    <row r="14" ht="43.2" customHeight="1">
       <c r="A14" s="225" t="n">
         <v>5</v>
       </c>
@@ -45793,7 +45790,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="26" customHeight="1">
+    <row r="15" ht="31.8" customHeight="1">
       <c r="A15" s="231" t="n">
         <v>6</v>
       </c>
@@ -45848,7 +45845,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="37" customHeight="1">
+    <row r="16" ht="43.2" customHeight="1">
       <c r="A16" s="225" t="n">
         <v>7</v>
       </c>
@@ -45903,7 +45900,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="37" customHeight="1">
+    <row r="17" ht="43.2" customHeight="1">
       <c r="A17" s="231" t="n">
         <v>8</v>
       </c>
@@ -45958,7 +45955,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="37" customHeight="1">
+    <row r="18" ht="54.6" customHeight="1">
       <c r="A18" s="225" t="n">
         <v>9</v>
       </c>
@@ -46013,7 +46010,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="26" customHeight="1">
+    <row r="19" ht="43.2" customHeight="1">
       <c r="A19" s="231" t="n">
         <v>10</v>
       </c>
@@ -46068,7 +46065,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="26" customHeight="1">
+    <row r="20" ht="31.8" customHeight="1">
       <c r="A20" s="225" t="n">
         <v>11</v>
       </c>
@@ -46178,7 +46175,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="26" customHeight="1">
+    <row r="22" ht="31.8" customHeight="1">
       <c r="A22" s="225" t="n">
         <v>13</v>
       </c>
@@ -46233,7 +46230,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="37" customHeight="1">
+    <row r="23" ht="43.2" customHeight="1">
       <c r="A23" s="231" t="n">
         <v>14</v>
       </c>
@@ -46288,7 +46285,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="26" customHeight="1">
+    <row r="24" ht="31.8" customHeight="1">
       <c r="A24" s="225" t="n">
         <v>15</v>
       </c>
@@ -46343,7 +46340,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="26" customHeight="1">
+    <row r="25" ht="31.8" customHeight="1">
       <c r="A25" s="231" t="n">
         <v>16</v>
       </c>
@@ -46398,7 +46395,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="26" customHeight="1">
+    <row r="26" ht="31.8" customHeight="1">
       <c r="A26" s="225" t="n">
         <v>17</v>
       </c>
@@ -46600,7 +46597,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="37" customHeight="1">
+    <row r="32" ht="54.6" customHeight="1">
       <c r="A32" s="243" t="inlineStr">
         <is>
           <t>R1</t>
@@ -46658,7 +46655,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="26" customHeight="1">
+    <row r="33" ht="31.8" customHeight="1">
       <c r="A33" s="249" t="inlineStr">
         <is>
           <t>R2</t>
@@ -46716,7 +46713,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="48" customHeight="1">
+    <row r="34" ht="77.40000000000001" customHeight="1">
       <c r="A34" s="243" t="inlineStr">
         <is>
           <t>R3</t>
@@ -46774,7 +46771,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="26" customHeight="1">
+    <row r="35" ht="31.8" customHeight="1">
       <c r="A35" s="249" t="inlineStr">
         <is>
           <t>R4</t>
@@ -47519,7 +47516,7 @@
       <c r="J53" s="6" t="n"/>
       <c r="K53" s="6" t="n"/>
     </row>
-    <row r="54" ht="30" customHeight="1">
+    <row r="54" ht="34" customHeight="1">
       <c r="A54" s="260" t="inlineStr">
         <is>
           <t>ID</t>
@@ -47537,7 +47534,7 @@
       </c>
       <c r="D54" s="260" t="inlineStr">
         <is>
-          <t>Finding (continued)</t>
+          <t>Finding (cont.)</t>
         </is>
       </c>
       <c r="E54" s="260" t="inlineStr">
@@ -47547,36 +47544,36 @@
       </c>
       <c r="F54" s="260" t="inlineStr">
         <is>
-          <t>Evidence (continued)</t>
+          <t>Evidence (cont.)</t>
         </is>
       </c>
       <c r="G54" s="260" t="inlineStr">
         <is>
+          <t>Evidence (cont.)</t>
+        </is>
+      </c>
+      <c r="H54" s="260" t="inlineStr">
+        <is>
           <t>Why it explains the reported result</t>
         </is>
       </c>
-      <c r="H54" s="260" t="inlineStr">
-        <is>
-          <t>Why it explains the reported result (continued)</t>
-        </is>
-      </c>
       <c r="I54" s="260" t="inlineStr">
         <is>
-          <t>Correction</t>
+          <t>Why it explains the reported result (cont.)</t>
         </is>
       </c>
       <c r="J54" s="260" t="inlineStr">
         <is>
-          <t>Correction (continued)</t>
+          <t>Correction  —  and the phase it goes to</t>
         </is>
       </c>
       <c r="K54" s="260" t="inlineStr">
         <is>
-          <t>Goes to</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="57" customHeight="1">
+          <t>Correction (cont.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="66" customHeight="1">
       <c r="A55" s="261" t="inlineStr">
         <is>
           <t>F-01</t>
@@ -47599,25 +47596,22 @@
         </is>
       </c>
       <c r="F55" s="263" t="n"/>
-      <c r="G55" s="237" t="inlineStr">
+      <c r="G55" s="263" t="n"/>
+      <c r="H55" s="237" t="inlineStr">
         <is>
           <t>SRS-based weights and beam tracking are the two bits that actually move DL MCS and DL user throughput. What did land was the interference / pairing-gate package, which does not add throughput on its own. The trial therefore did not test the DL hypothesis at all.</t>
         </is>
       </c>
-      <c r="H55" s="263" t="n"/>
-      <c r="I55" s="264" t="inlineStr">
-        <is>
-          <t>Ph2: send DlCoverageAlgoSwitch=SUPER_COVERAGE_SW-1 first, then the four beam bits one per MML line. Only then re-measure DL user throughput.</t>
-        </is>
-      </c>
-      <c r="J55" s="263" t="n"/>
-      <c r="K55" s="265" t="inlineStr">
-        <is>
-          <t>Ph2  step 2.2 → 2.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="57" customHeight="1">
+      <c r="I55" s="263" t="n"/>
+      <c r="J55" s="264" t="inlineStr">
+        <is>
+          <t>Ph2: send DlCoverageAlgoSwitch=SUPER_COVERAGE_SW-1 first, then the four beam bits one per MML line. Only then re-measure DL user throughput.
+→  Goes to:  Ph2 steps 2.2 → 2.6</t>
+        </is>
+      </c>
+      <c r="K55" s="263" t="n"/>
+    </row>
+    <row r="56" ht="66" customHeight="1">
       <c r="A56" s="261" t="inlineStr">
         <is>
           <t>F-02</t>
@@ -47640,31 +47634,28 @@
         </is>
       </c>
       <c r="F56" s="263" t="n"/>
-      <c r="G56" s="237" t="inlineStr">
+      <c r="G56" s="263" t="n"/>
+      <c r="H56" s="237" t="inlineStr">
         <is>
           <t>Both switches change how SRS is detected and multiplexed. Together the SRS channel estimate degrades, and everything downstream of SRS — DL weights, MU pairing eligibility, UL rank — degrades with it. This is the most likely direct cause of the pairing collapse.</t>
         </is>
       </c>
-      <c r="H56" s="263" t="n"/>
-      <c r="I56" s="264" t="inlineStr">
-        <is>
-          <t>Ph2 night 1, single change: SRS_IC_SW-0. Keep tight multiplexing. Confirm with N.SRS.NI.Avg and N.UL.SRS.PreSINR.Index* over 9–12 Sep.</t>
-        </is>
-      </c>
-      <c r="J56" s="263" t="n"/>
-      <c r="K56" s="265" t="inlineStr">
-        <is>
-          <t>Ph2  step 2.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="57" customHeight="1">
-      <c r="A57" s="266" t="inlineStr">
+      <c r="I56" s="263" t="n"/>
+      <c r="J56" s="264" t="inlineStr">
+        <is>
+          <t>Ph2 night 1, single change: SRS_IC_SW-0. Keep tight multiplexing. Confirm with N.SRS.NI.Avg and N.UL.SRS.PreSINR.Index* over 9–12 Sep.
+→  Goes to:  Ph2 step 2.1</t>
+        </is>
+      </c>
+      <c r="K56" s="263" t="n"/>
+    </row>
+    <row r="57" ht="54.6" customHeight="1">
+      <c r="A57" s="265" t="inlineStr">
         <is>
           <t>F-03</t>
         </is>
       </c>
-      <c r="B57" s="267" t="inlineStr">
+      <c r="B57" s="266" t="inlineStr">
         <is>
           <t>MAJOR</t>
         </is>
@@ -47681,31 +47672,28 @@
         </is>
       </c>
       <c r="F57" s="263" t="n"/>
-      <c r="G57" s="237" t="inlineStr">
+      <c r="G57" s="263" t="n"/>
+      <c r="H57" s="237" t="inlineStr">
         <is>
           <t>Both switches are quality gates — they reject pairs whose channel estimate is not clean. Fed with degraded SRS they reject almost everything, so paired RB falls. The pairing drop is the two findings above acting together, not a defect in either feature.</t>
         </is>
       </c>
-      <c r="H57" s="263" t="n"/>
-      <c r="I57" s="264" t="inlineStr">
-        <is>
-          <t>Do not roll these back first. Fix SRS (F-02), re-measure, and only then decide — one switch per night, 24 h apart.</t>
-        </is>
-      </c>
-      <c r="J57" s="263" t="n"/>
-      <c r="K57" s="265" t="inlineStr">
-        <is>
-          <t>Ph3  night 1–2</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="57" customHeight="1">
-      <c r="A58" s="266" t="inlineStr">
+      <c r="I57" s="263" t="n"/>
+      <c r="J57" s="264" t="inlineStr">
+        <is>
+          <t>Do not roll these back first. Fix SRS (F-02), re-measure, and only then decide — one switch per night, 24 h apart.
+→  Goes to:  Ph3 nights 1–2</t>
+        </is>
+      </c>
+      <c r="K57" s="263" t="n"/>
+    </row>
+    <row r="58" ht="54.6" customHeight="1">
+      <c r="A58" s="265" t="inlineStr">
         <is>
           <t>F-04</t>
         </is>
       </c>
-      <c r="B58" s="267" t="inlineStr">
+      <c r="B58" s="266" t="inlineStr">
         <is>
           <t>MAJOR</t>
         </is>
@@ -47722,31 +47710,28 @@
         </is>
       </c>
       <c r="F58" s="263" t="n"/>
-      <c r="G58" s="237" t="inlineStr">
+      <c r="G58" s="263" t="n"/>
+      <c r="H58" s="237" t="inlineStr">
         <is>
           <t>Ph1 contained only gates that can reduce pairing and no feature that can add layers. Even with healthy SRS, N.ChMeas.MIMO.DL.MuPairing.4…16Layer.RB had no mechanism to rise.</t>
         </is>
       </c>
-      <c r="H58" s="263" t="n"/>
-      <c r="I58" s="264" t="inlineStr">
-        <is>
-          <t>Ph4: enable HighLayerMuMimoSw=MMIMO_MULTILAYER_ENHANCE_SW-1 as the master, then its children one per night. That is the phase that is supposed to spend the LAYER_16 quota.</t>
-        </is>
-      </c>
-      <c r="J58" s="263" t="n"/>
-      <c r="K58" s="265" t="inlineStr">
-        <is>
-          <t>Ph4</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="57" customHeight="1">
-      <c r="A59" s="266" t="inlineStr">
+      <c r="I58" s="263" t="n"/>
+      <c r="J58" s="264" t="inlineStr">
+        <is>
+          <t>Ph4: enable HighLayerMuMimoSw=MMIMO_MULTILAYER_ENHANCE_SW-1 as the master, then its children one per night. That is the phase that is supposed to spend the LAYER_16 quota.
+→  Goes to:  Ph4</t>
+        </is>
+      </c>
+      <c r="K58" s="263" t="n"/>
+    </row>
+    <row r="59" ht="54.6" customHeight="1">
+      <c r="A59" s="265" t="inlineStr">
         <is>
           <t>F-05</t>
         </is>
       </c>
-      <c r="B59" s="267" t="inlineStr">
+      <c r="B59" s="266" t="inlineStr">
         <is>
           <t>MAJOR</t>
         </is>
@@ -47763,36 +47748,33 @@
         </is>
       </c>
       <c r="F59" s="263" t="n"/>
-      <c r="G59" s="237" t="inlineStr">
+      <c r="G59" s="263" t="n"/>
+      <c r="H59" s="237" t="inlineStr">
         <is>
           <t>One invalid option rejects the entire command, so three healthy switches were lost with the one that had a missing pre-requisite. It also makes the result impossible to attribute: when a KPI moves, nobody can say which bit moved it.</t>
         </is>
       </c>
-      <c r="H59" s="263" t="n"/>
-      <c r="I59" s="264" t="inlineStr">
-        <is>
-          <t>Execution rule from v7.0 onward: one switch per MML line, in the sequence given by the new pre-requisite columns on sheet 14. Sheet 17 Ph2 is written that way.</t>
-        </is>
-      </c>
-      <c r="J59" s="263" t="n"/>
-      <c r="K59" s="265" t="inlineStr">
-        <is>
-          <t>Sheet 14 pre-req columns + sheet 17 golden rules</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="57" customHeight="1">
-      <c r="A60" s="268" t="inlineStr">
+      <c r="I59" s="263" t="n"/>
+      <c r="J59" s="264" t="inlineStr">
+        <is>
+          <t>Execution rule from v7.0 onward: one switch per MML line, in the sequence given by the new pre-requisite columns on sheet 14. Sheet 17 Ph2 is written that way.
+→  Goes to:  Sheet 14 pre-requisite columns + sheet 17 Section 4</t>
+        </is>
+      </c>
+      <c r="K59" s="263" t="n"/>
+    </row>
+    <row r="60" ht="54.6" customHeight="1">
+      <c r="A60" s="267" t="inlineStr">
         <is>
           <t>F-06</t>
         </is>
       </c>
-      <c r="B60" s="269" t="inlineStr">
+      <c r="B60" s="268" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="C60" s="270" t="inlineStr">
+      <c r="C60" s="269" t="inlineStr">
         <is>
           <t>The real execution window is 10–11 Sep 2026, not 11 Sep only</t>
         </is>
@@ -47804,36 +47786,33 @@
         </is>
       </c>
       <c r="F60" s="263" t="n"/>
-      <c r="G60" s="237" t="inlineStr">
+      <c r="G60" s="263" t="n"/>
+      <c r="H60" s="237" t="inlineStr">
         <is>
           <t>Using 11 Sep as the only execution date makes 10 Sep look like a valid baseline day, which would understate the regression by roughly a third.</t>
         </is>
       </c>
-      <c r="H60" s="263" t="n"/>
-      <c r="I60" s="264" t="inlineStr">
-        <is>
-          <t>Use 5 Sep and 9 Sep as the baseline, 10–11 Sep as the execution window and 12 Sep as D+1 in every comparison from now on.</t>
-        </is>
-      </c>
-      <c r="J60" s="263" t="n"/>
-      <c r="K60" s="265" t="inlineStr">
-        <is>
-          <t>All future baselines</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="44" customHeight="1">
-      <c r="A61" s="268" t="inlineStr">
+      <c r="I60" s="263" t="n"/>
+      <c r="J60" s="264" t="inlineStr">
+        <is>
+          <t>Use 5 Sep and 9 Sep as the baseline, 10–11 Sep as the execution window and 12 Sep as D+1 in every comparison from now on.
+→  Goes to:  Every future baseline</t>
+        </is>
+      </c>
+      <c r="K60" s="263" t="n"/>
+    </row>
+    <row r="61" ht="43.2" customHeight="1">
+      <c r="A61" s="267" t="inlineStr">
         <is>
           <t>F-07</t>
         </is>
       </c>
-      <c r="B61" s="269" t="inlineStr">
+      <c r="B61" s="268" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="C61" s="270" t="inlineStr">
+      <c r="C61" s="269" t="inlineStr">
         <is>
           <t>12 Sep recovers part of the loss but stays well below baseline — it is not self-healing</t>
         </is>
@@ -47845,36 +47824,33 @@
         </is>
       </c>
       <c r="F61" s="263" t="n"/>
-      <c r="G61" s="237" t="inlineStr">
+      <c r="G61" s="263" t="n"/>
+      <c r="H61" s="237" t="inlineStr">
         <is>
           <t>Part of the 11 Sep dip is load or transient, but 12 Sep is still 41 % down. Waiting will not close the gap, so a configuration change is required.</t>
         </is>
       </c>
-      <c r="H61" s="263" t="n"/>
-      <c r="I61" s="264" t="inlineStr">
-        <is>
-          <t>Do not wait for further recovery. Run Ph2 at the next maintenance window.</t>
-        </is>
-      </c>
-      <c r="J61" s="263" t="n"/>
-      <c r="K61" s="265" t="inlineStr">
-        <is>
-          <t>Ph2 scheduling</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="57" customHeight="1">
-      <c r="A62" s="268" t="inlineStr">
+      <c r="I61" s="263" t="n"/>
+      <c r="J61" s="264" t="inlineStr">
+        <is>
+          <t>Do not wait for further recovery. Run Ph2 at the next maintenance window.
+→  Goes to:  Ph2 scheduling</t>
+        </is>
+      </c>
+      <c r="K61" s="263" t="n"/>
+    </row>
+    <row r="62" ht="54.6" customHeight="1">
+      <c r="A62" s="267" t="inlineStr">
         <is>
           <t>F-08</t>
         </is>
       </c>
-      <c r="B62" s="269" t="inlineStr">
+      <c r="B62" s="268" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="C62" s="270" t="inlineStr">
+      <c r="C62" s="269" t="inlineStr">
         <is>
           <t>Evidence gap: the counters that would prove the root cause were not supplied</t>
         </is>
@@ -47886,23 +47862,20 @@
         </is>
       </c>
       <c r="F62" s="263" t="n"/>
-      <c r="G62" s="237" t="inlineStr">
+      <c r="G62" s="263" t="n"/>
+      <c r="H62" s="237" t="inlineStr">
         <is>
           <t>Without SRS NI the SRS_IC conflict stays a strong hypothesis. Without PRB load the pairing drop cannot be separated from a simple traffic change. Without IBLER it is unknown whether the stricter gates bought quality for the RB they gave up.</t>
         </is>
       </c>
-      <c r="H62" s="263" t="n"/>
-      <c r="I62" s="264" t="inlineStr">
-        <is>
-          <t>Pull N.SRS.NI.Avg, N.UL.SRS.PreSINR.Index*, DL IBLER, N.CCE.Used.Avg and N.PRB.DL.Used.Avg for 5–12 Sep, trial and neighbour control, before Ph2 sign-off.</t>
-        </is>
-      </c>
-      <c r="J62" s="263" t="n"/>
-      <c r="K62" s="265" t="inlineStr">
-        <is>
-          <t>Counter pull before Ph2</t>
-        </is>
-      </c>
+      <c r="I62" s="263" t="n"/>
+      <c r="J62" s="264" t="inlineStr">
+        <is>
+          <t>Pull N.SRS.NI.Avg, N.UL.SRS.PreSINR.Index*, DL IBLER, N.CCE.Used.Avg and N.PRB.DL.Used.Avg for 5–12 Sep, trial and neighbour control, before Ph2 sign-off.
+→  Goes to:  Counter pull before Ph2 sign-off</t>
+        </is>
+      </c>
+      <c r="K62" s="263" t="n"/>
     </row>
     <row r="63" ht="8" customHeight="1"/>
     <row r="64" ht="22" customHeight="1">
@@ -47922,68 +47895,68 @@
       <c r="J64" s="6" t="n"/>
       <c r="K64" s="6" t="n"/>
     </row>
-    <row r="65" ht="30" customHeight="1">
-      <c r="A65" s="271" t="inlineStr">
+    <row r="65" ht="34" customHeight="1">
+      <c r="A65" s="270" t="inlineStr">
         <is>
           <t>SN</t>
         </is>
       </c>
-      <c r="B65" s="271" t="inlineStr">
+      <c r="B65" s="270" t="inlineStr">
         <is>
           <t>Rule in the workbook</t>
         </is>
       </c>
-      <c r="C65" s="271" t="inlineStr">
-        <is>
-          <t>Rule in the workbook (continued)</t>
-        </is>
-      </c>
-      <c r="D65" s="271" t="inlineStr">
+      <c r="C65" s="270" t="inlineStr">
+        <is>
+          <t>Rule (cont.)</t>
+        </is>
+      </c>
+      <c r="D65" s="270" t="inlineStr">
         <is>
           <t>What the Ph1 work order did instead</t>
         </is>
       </c>
-      <c r="E65" s="271" t="inlineStr">
-        <is>
-          <t>What the Ph1 work order did instead (continued)</t>
-        </is>
-      </c>
-      <c r="F65" s="271" t="inlineStr">
+      <c r="E65" s="270" t="inlineStr">
+        <is>
+          <t>(cont.)</t>
+        </is>
+      </c>
+      <c r="F65" s="270" t="inlineStr">
         <is>
           <t>Consequence</t>
         </is>
       </c>
-      <c r="G65" s="271" t="inlineStr">
-        <is>
-          <t>Consequence (continued)</t>
-        </is>
-      </c>
-      <c r="H65" s="271" t="inlineStr">
+      <c r="G65" s="270" t="inlineStr">
+        <is>
+          <t>Consequence (cont.)</t>
+        </is>
+      </c>
+      <c r="H65" s="270" t="inlineStr">
+        <is>
+          <t>Consequence (cont.)</t>
+        </is>
+      </c>
+      <c r="I65" s="270" t="inlineStr">
         <is>
           <t>Fix now in place</t>
         </is>
       </c>
-      <c r="I65" s="271" t="inlineStr">
-        <is>
-          <t>Fix now in place (continued)</t>
-        </is>
-      </c>
-      <c r="J65" s="271" t="inlineStr">
-        <is>
-          <t>Where</t>
-        </is>
-      </c>
-      <c r="K65" s="271" t="inlineStr">
-        <is>
-          <t>Where (continued)</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="40" customHeight="1">
-      <c r="A66" s="272" t="n">
+      <c r="J65" s="270" t="inlineStr">
+        <is>
+          <t>Fix (cont.)</t>
+        </is>
+      </c>
+      <c r="K65" s="270" t="inlineStr">
+        <is>
+          <t>Where to find it</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="31.8" customHeight="1">
+      <c r="A66" s="271" t="n">
         <v>1</v>
       </c>
-      <c r="B66" s="273" t="inlineStr">
+      <c r="B66" s="272" t="inlineStr">
         <is>
           <t>Send one parameter / one switch per MML line.</t>
         </is>
@@ -48001,24 +47974,24 @@
         </is>
       </c>
       <c r="G66" s="263" t="n"/>
-      <c r="H66" s="248" t="inlineStr">
+      <c r="H66" s="263" t="n"/>
+      <c r="I66" s="248" t="inlineStr">
         <is>
           <t>Sheet 17 Ph2 is written as seven separately numbered MML lines, one switch each.</t>
         </is>
       </c>
-      <c r="I66" s="263" t="n"/>
-      <c r="J66" s="227" t="inlineStr">
+      <c r="J66" s="263" t="n"/>
+      <c r="K66" s="227" t="inlineStr">
         <is>
           <t>Sheet 17 Section 2</t>
         </is>
       </c>
-      <c r="K66" s="263" t="n"/>
-    </row>
-    <row r="67" ht="52" customHeight="1">
-      <c r="A67" s="274" t="n">
+    </row>
+    <row r="67" ht="31.8" customHeight="1">
+      <c r="A67" s="273" t="n">
         <v>2</v>
       </c>
-      <c r="B67" s="273" t="inlineStr">
+      <c r="B67" s="272" t="inlineStr">
         <is>
           <t>Check the dependent switch before writing the work order.</t>
         </is>
@@ -48036,24 +48009,24 @@
         </is>
       </c>
       <c r="G67" s="263" t="n"/>
-      <c r="H67" s="248" t="inlineStr">
+      <c r="H67" s="263" t="n"/>
+      <c r="I67" s="248" t="inlineStr">
         <is>
           <t>Every MML row on sheet 14 now carries its pre-requisite switch and the exact pre-requisite MML to run before it.</t>
         </is>
       </c>
-      <c r="I67" s="263" t="n"/>
-      <c r="J67" s="233" t="inlineStr">
+      <c r="J67" s="263" t="n"/>
+      <c r="K67" s="233" t="inlineStr">
         <is>
           <t>Sheet 14, the two red columns</t>
         </is>
       </c>
-      <c r="K67" s="263" t="n"/>
-    </row>
-    <row r="68" ht="52" customHeight="1">
-      <c r="A68" s="272" t="n">
+    </row>
+    <row r="68" ht="31.8" customHeight="1">
+      <c r="A68" s="271" t="n">
         <v>3</v>
       </c>
-      <c r="B68" s="273" t="inlineStr">
+      <c r="B68" s="272" t="inlineStr">
         <is>
           <t>Do not enable SRS_IC the same night as SRS_TIGHT_MULTIPLEXING.</t>
         </is>
@@ -48071,24 +48044,24 @@
         </is>
       </c>
       <c r="G68" s="263" t="n"/>
-      <c r="H68" s="248" t="inlineStr">
+      <c r="H68" s="263" t="n"/>
+      <c r="I68" s="248" t="inlineStr">
         <is>
           <t>SRS_IC_SW-0 is Ph2 step 2.1 and it is the ONLY change that night.</t>
         </is>
       </c>
-      <c r="I68" s="263" t="n"/>
-      <c r="J68" s="227" t="inlineStr">
+      <c r="J68" s="263" t="n"/>
+      <c r="K68" s="227" t="inlineStr">
         <is>
           <t>Sheet 17 Ph2 step 2.1</t>
         </is>
       </c>
-      <c r="K68" s="263" t="n"/>
-    </row>
-    <row r="69" ht="52" customHeight="1">
-      <c r="A69" s="274" t="n">
+    </row>
+    <row r="69" ht="31.8" customHeight="1">
+      <c r="A69" s="273" t="n">
         <v>4</v>
       </c>
-      <c r="B69" s="273" t="inlineStr">
+      <c r="B69" s="272" t="inlineStr">
         <is>
           <t>Verify each line with an LST and keep the RETCODE.</t>
         </is>
@@ -48106,24 +48079,24 @@
         </is>
       </c>
       <c r="G69" s="263" t="n"/>
-      <c r="H69" s="248" t="inlineStr">
+      <c r="H69" s="263" t="n"/>
+      <c r="I69" s="248" t="inlineStr">
         <is>
           <t>Every Ph2 step now has its own Verify (LST) column and must return RETCODE = 0 before the next step is sent.</t>
         </is>
       </c>
-      <c r="I69" s="263" t="n"/>
-      <c r="J69" s="233" t="inlineStr">
+      <c r="J69" s="263" t="n"/>
+      <c r="K69" s="233" t="inlineStr">
         <is>
           <t>Sheet 17 Ph2, Verify column</t>
         </is>
       </c>
-      <c r="K69" s="263" t="n"/>
-    </row>
-    <row r="70" ht="52" customHeight="1">
-      <c r="A70" s="272" t="n">
+    </row>
+    <row r="70" ht="31.8" customHeight="1">
+      <c r="A70" s="271" t="n">
         <v>5</v>
       </c>
-      <c r="B70" s="273" t="inlineStr">
+      <c r="B70" s="272" t="inlineStr">
         <is>
           <t>One root cause per maintenance night.</t>
         </is>
@@ -48141,18 +48114,18 @@
         </is>
       </c>
       <c r="G70" s="263" t="n"/>
-      <c r="H70" s="248" t="inlineStr">
+      <c r="H70" s="263" t="n"/>
+      <c r="I70" s="248" t="inlineStr">
         <is>
           <t>Ph2 to Ph7 are one family per phase and one switch per night, each with its own exit gate.</t>
         </is>
       </c>
-      <c r="I70" s="263" t="n"/>
-      <c r="J70" s="227" t="inlineStr">
+      <c r="J70" s="263" t="n"/>
+      <c r="K70" s="227" t="inlineStr">
         <is>
           <t>Sheet 17 Section 1</t>
         </is>
       </c>
-      <c r="K70" s="263" t="n"/>
     </row>
     <row r="71" ht="8" customHeight="1"/>
     <row r="72" ht="22" customHeight="1">
@@ -48173,7 +48146,7 @@
       <c r="K72" s="6" t="n"/>
     </row>
     <row r="73" ht="118" customHeight="1">
-      <c r="A73" s="275" t="inlineStr">
+      <c r="A73" s="274" t="inlineStr">
         <is>
           <t>•  N.SRS.NI.Avg and N.UL.SRS.PreSINR.Index*, 5–12 Sep, trial and control — the only data that turns finding F-02 from a strong hypothesis into proof.
 •  DL IBLER (Σ N.DL.SCH.*.ErrTB.Ibler / Σ N.DL.SCH.*.TB) — tells whether the stricter MU gates bought link quality for the paired RB they gave up. If IBLER improved, the gates are working as designed and only the SRS input was bad.
@@ -48183,16 +48156,16 @@
 •  The full MML execution log for 10 and 11 Sep with every RETCODE, not only the one failure — there may be further silent rejections in the same work order.</t>
         </is>
       </c>
-      <c r="B73" s="276" t="n"/>
-      <c r="C73" s="276" t="n"/>
-      <c r="D73" s="276" t="n"/>
-      <c r="E73" s="276" t="n"/>
-      <c r="F73" s="276" t="n"/>
-      <c r="G73" s="276" t="n"/>
-      <c r="H73" s="276" t="n"/>
-      <c r="I73" s="276" t="n"/>
-      <c r="J73" s="276" t="n"/>
-      <c r="K73" s="276" t="n"/>
+      <c r="B73" s="275" t="n"/>
+      <c r="C73" s="275" t="n"/>
+      <c r="D73" s="275" t="n"/>
+      <c r="E73" s="275" t="n"/>
+      <c r="F73" s="275" t="n"/>
+      <c r="G73" s="275" t="n"/>
+      <c r="H73" s="275" t="n"/>
+      <c r="I73" s="275" t="n"/>
+      <c r="J73" s="275" t="n"/>
+      <c r="K73" s="275" t="n"/>
     </row>
     <row r="75" ht="12" customHeight="1"/>
     <row r="76" ht="22" customHeight="1">
@@ -48787,87 +48760,82 @@
       <c r="K95" s="151" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="80">
+  <mergeCells count="75">
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="E94:J94"/>
     <mergeCell ref="C62:D62"/>
-    <mergeCell ref="E62:F62"/>
+    <mergeCell ref="A30:K30"/>
+    <mergeCell ref="A77:K77"/>
+    <mergeCell ref="E60:G60"/>
     <mergeCell ref="A64:K64"/>
-    <mergeCell ref="F68:G68"/>
+    <mergeCell ref="C58:D58"/>
     <mergeCell ref="A73:K73"/>
     <mergeCell ref="A51:K51"/>
-    <mergeCell ref="J68:K68"/>
+    <mergeCell ref="J57:K57"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="F70:H70"/>
+    <mergeCell ref="H55:I55"/>
+    <mergeCell ref="J59:K59"/>
+    <mergeCell ref="F66:H66"/>
+    <mergeCell ref="H58:I58"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="E59:G59"/>
+    <mergeCell ref="J60:K60"/>
+    <mergeCell ref="I70:J70"/>
+    <mergeCell ref="H56:I56"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="H59:I59"/>
+    <mergeCell ref="E95:J95"/>
     <mergeCell ref="A7:K7"/>
+    <mergeCell ref="H60:I60"/>
     <mergeCell ref="B67:C67"/>
-    <mergeCell ref="G57:H57"/>
+    <mergeCell ref="E61:G61"/>
+    <mergeCell ref="C55:D55"/>
+    <mergeCell ref="E91:J91"/>
+    <mergeCell ref="E57:G57"/>
+    <mergeCell ref="I66:J66"/>
+    <mergeCell ref="H61:I61"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="J55:K55"/>
+    <mergeCell ref="C56:D56"/>
+    <mergeCell ref="A37:K37"/>
+    <mergeCell ref="F67:H67"/>
     <mergeCell ref="D70:E70"/>
-    <mergeCell ref="F70:G70"/>
-    <mergeCell ref="C56:D56"/>
-    <mergeCell ref="I58:J58"/>
+    <mergeCell ref="C59:D59"/>
+    <mergeCell ref="A89:K89"/>
     <mergeCell ref="B69:C69"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="G58:H58"/>
-    <mergeCell ref="A53:K53"/>
-    <mergeCell ref="G59:H59"/>
-    <mergeCell ref="A30:K30"/>
-    <mergeCell ref="E55:F55"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="G61:H61"/>
-    <mergeCell ref="I61:J61"/>
-    <mergeCell ref="H68:I68"/>
-    <mergeCell ref="I57:J57"/>
-    <mergeCell ref="G62:H62"/>
-    <mergeCell ref="E91:J91"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="I56:J56"/>
-    <mergeCell ref="F66:G66"/>
-    <mergeCell ref="H69:I69"/>
+    <mergeCell ref="I68:J68"/>
+    <mergeCell ref="I69:J69"/>
     <mergeCell ref="C60:D60"/>
     <mergeCell ref="E93:J93"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="I67:J67"/>
+    <mergeCell ref="E56:G56"/>
+    <mergeCell ref="H57:I57"/>
+    <mergeCell ref="E58:G58"/>
+    <mergeCell ref="C61:D61"/>
     <mergeCell ref="A76:K76"/>
+    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="F69:H69"/>
     <mergeCell ref="A8:K8"/>
-    <mergeCell ref="C57:D57"/>
-    <mergeCell ref="I59:J59"/>
-    <mergeCell ref="G60:H60"/>
-    <mergeCell ref="E58:F58"/>
-    <mergeCell ref="I60:J60"/>
-    <mergeCell ref="C58:D58"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A37:K37"/>
-    <mergeCell ref="C59:D59"/>
-    <mergeCell ref="A89:K89"/>
-    <mergeCell ref="E59:F59"/>
-    <mergeCell ref="I62:J62"/>
-    <mergeCell ref="C61:D61"/>
-    <mergeCell ref="E61:F61"/>
-    <mergeCell ref="H66:I66"/>
-    <mergeCell ref="J66:K66"/>
-    <mergeCell ref="E57:F57"/>
+    <mergeCell ref="J56:K56"/>
+    <mergeCell ref="E55:G55"/>
+    <mergeCell ref="A53:K53"/>
+    <mergeCell ref="E62:G62"/>
+    <mergeCell ref="B68:C68"/>
     <mergeCell ref="A4:K4"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="E92:J92"/>
-    <mergeCell ref="E56:F56"/>
-    <mergeCell ref="G56:H56"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="H67:I67"/>
-    <mergeCell ref="F69:G69"/>
-    <mergeCell ref="E94:J94"/>
-    <mergeCell ref="J67:K67"/>
-    <mergeCell ref="A77:K77"/>
-    <mergeCell ref="J69:K69"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="E95:J95"/>
-    <mergeCell ref="C55:D55"/>
-    <mergeCell ref="E60:F60"/>
-    <mergeCell ref="H70:I70"/>
-    <mergeCell ref="J70:K70"/>
-    <mergeCell ref="I55:J55"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="F67:G67"/>
-    <mergeCell ref="G55:H55"/>
-    <mergeCell ref="B68:C68"/>
     <mergeCell ref="D68:E68"/>
+    <mergeCell ref="F68:H68"/>
     <mergeCell ref="A72:K72"/>
     <mergeCell ref="A29:K29"/>
+    <mergeCell ref="H62:I62"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="C57:D57"/>
     <mergeCell ref="A38:K38"/>
+    <mergeCell ref="J62:K62"/>
+    <mergeCell ref="E92:J92"/>
+    <mergeCell ref="J61:K61"/>
+    <mergeCell ref="J58:K58"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.5" header="0.25" footer="0.25"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -48893,34 +48861,34 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="31" customWidth="1" min="4" max="4"/>
-    <col width="37" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="277" t="inlineStr">
+      <c r="A1" s="276" t="inlineStr">
         <is>
           <t xml:space="preserve">  Action Plan  —  Ph1 complete,  Ph2 corrective,  Ph3…Ph7 staged</t>
         </is>
       </c>
-      <c r="B1" s="278" t="n"/>
-      <c r="C1" s="278" t="n"/>
-      <c r="D1" s="278" t="n"/>
-      <c r="E1" s="278" t="n"/>
-      <c r="F1" s="278" t="n"/>
-      <c r="G1" s="278" t="n"/>
-      <c r="H1" s="278" t="n"/>
-      <c r="I1" s="278" t="n"/>
-      <c r="J1" s="278" t="n"/>
-      <c r="K1" s="278" t="n"/>
+      <c r="B1" s="277" t="n"/>
+      <c r="C1" s="277" t="n"/>
+      <c r="D1" s="277" t="n"/>
+      <c r="E1" s="277" t="n"/>
+      <c r="F1" s="277" t="n"/>
+      <c r="G1" s="277" t="n"/>
+      <c r="H1" s="277" t="n"/>
+      <c r="I1" s="277" t="n"/>
+      <c r="J1" s="277" t="n"/>
+      <c r="K1" s="277" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="16" t="inlineStr">
@@ -48941,92 +48909,92 @@
     </row>
     <row r="3" ht="6" customHeight="1"/>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="279" t="inlineStr">
+      <c r="A4" s="278" t="inlineStr">
         <is>
           <t>Section 1.  Phase overview</t>
         </is>
       </c>
-      <c r="B4" s="280" t="n"/>
-      <c r="C4" s="280" t="n"/>
-      <c r="D4" s="280" t="n"/>
-      <c r="E4" s="280" t="n"/>
-      <c r="F4" s="280" t="n"/>
-      <c r="G4" s="280" t="n"/>
-      <c r="H4" s="280" t="n"/>
-      <c r="I4" s="280" t="n"/>
-      <c r="J4" s="280" t="n"/>
-      <c r="K4" s="280" t="n"/>
+      <c r="B4" s="279" t="n"/>
+      <c r="C4" s="279" t="n"/>
+      <c r="D4" s="279" t="n"/>
+      <c r="E4" s="279" t="n"/>
+      <c r="F4" s="279" t="n"/>
+      <c r="G4" s="279" t="n"/>
+      <c r="H4" s="279" t="n"/>
+      <c r="I4" s="279" t="n"/>
+      <c r="J4" s="279" t="n"/>
+      <c r="K4" s="279" t="n"/>
     </row>
     <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="281" t="inlineStr">
+      <c r="A5" s="280" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B5" s="281" t="inlineStr">
+      <c r="B5" s="280" t="inlineStr">
         <is>
           <t>Window</t>
         </is>
       </c>
-      <c r="C5" s="281" t="inlineStr">
+      <c r="C5" s="280" t="inlineStr">
         <is>
           <t>Objective</t>
         </is>
       </c>
-      <c r="D5" s="281" t="inlineStr">
+      <c r="D5" s="280" t="inlineStr">
         <is>
           <t>Content  (one switch per MML line)</t>
         </is>
       </c>
-      <c r="E5" s="281" t="inlineStr">
+      <c r="E5" s="280" t="inlineStr">
         <is>
           <t>Pre-requisite to verify BEFORE the work order is written</t>
         </is>
       </c>
-      <c r="F5" s="281" t="inlineStr">
+      <c r="F5" s="280" t="inlineStr">
         <is>
           <t>Pre-requisite to verify (continued)</t>
         </is>
       </c>
-      <c r="G5" s="281" t="inlineStr">
+      <c r="G5" s="280" t="inlineStr">
         <is>
           <t>Exit KPI gate</t>
         </is>
       </c>
-      <c r="H5" s="281" t="inlineStr">
+      <c r="H5" s="280" t="inlineStr">
         <is>
           <t>Exit KPI gate (continued)</t>
         </is>
       </c>
-      <c r="I5" s="281" t="inlineStr">
+      <c r="I5" s="280" t="inlineStr">
         <is>
           <t>Rollback</t>
         </is>
       </c>
-      <c r="J5" s="281" t="inlineStr">
+      <c r="J5" s="280" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="K5" s="281" t="inlineStr">
+      <c r="K5" s="280" t="inlineStr">
         <is>
           <t>Status (continued)</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="75" customHeight="1">
-      <c r="A6" s="282" t="inlineStr">
+    <row r="6" ht="66" customHeight="1">
+      <c r="A6" s="281" t="inlineStr">
         <is>
           <t>Ph1</t>
         </is>
       </c>
-      <c r="B6" s="283" t="inlineStr">
+      <c r="B6" s="282" t="inlineStr">
         <is>
           <t>10–11 Sep 2026
 (done)</t>
         </is>
       </c>
-      <c r="C6" s="284" t="inlineStr">
+      <c r="C6" s="283" t="inlineStr">
         <is>
           <t>Land the SRS / UL Boosting / iBeam 1.0 interference package and the beam-weight levers.</t>
         </is>
@@ -49053,15 +49021,15 @@
           <t>Not required as a whole. Ph2 rolls back one switch (SRS_IC_SW) only.</t>
         </is>
       </c>
-      <c r="J6" s="285" t="inlineStr">
+      <c r="J6" s="284" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
       <c r="K6" s="263" t="n"/>
     </row>
-    <row r="7" ht="88" customHeight="1">
-      <c r="A7" s="286" t="inlineStr">
+    <row r="7" ht="88.8" customHeight="1">
+      <c r="A7" s="285" t="inlineStr">
         <is>
           <t>Ph2</t>
         </is>
@@ -49099,25 +49067,25 @@
           <t>Night 1: SRS_IC_SW-1 back. Night 2: the four beam bits back to 0, SUPER_COVERAGE_SW back to its pre-change value. Never touch HighPrecisionBeamSwitch.</t>
         </is>
       </c>
-      <c r="J7" s="287" t="inlineStr">
+      <c r="J7" s="286" t="inlineStr">
         <is>
           <t>NEXT</t>
         </is>
       </c>
       <c r="K7" s="263" t="n"/>
     </row>
-    <row r="8" ht="75" customHeight="1">
-      <c r="A8" s="288" t="inlineStr">
+    <row r="8" ht="77.40000000000001" customHeight="1">
+      <c r="A8" s="287" t="inlineStr">
         <is>
           <t>Ph3</t>
         </is>
       </c>
-      <c r="B8" s="289" t="inlineStr">
+      <c r="B8" s="288" t="inlineStr">
         <is>
           <t>Ph2 + 7 days</t>
         </is>
       </c>
-      <c r="C8" s="290" t="inlineStr">
+      <c r="C8" s="289" t="inlineStr">
         <is>
           <t>Decide the fate of the two DL MU quality gates, then add SSB beam adaptation.</t>
         </is>
@@ -49144,25 +49112,25 @@
           <t>Re-enable the rolled-back MU gate, or SSB_BEAM_ADAPT_SW-0 — whichever that night touched.</t>
         </is>
       </c>
-      <c r="J8" s="268" t="inlineStr">
+      <c r="J8" s="267" t="inlineStr">
         <is>
           <t>PLANNED</t>
         </is>
       </c>
       <c r="K8" s="263" t="n"/>
     </row>
-    <row r="9" ht="75" customHeight="1">
-      <c r="A9" s="288" t="inlineStr">
+    <row r="9" ht="66" customHeight="1">
+      <c r="A9" s="287" t="inlineStr">
         <is>
           <t>Ph4</t>
         </is>
       </c>
-      <c r="B9" s="289" t="inlineStr">
+      <c r="B9" s="288" t="inlineStr">
         <is>
           <t>Ph3 + 7 days</t>
         </is>
       </c>
-      <c r="C9" s="290" t="inlineStr">
+      <c r="C9" s="289" t="inlineStr">
         <is>
           <t>Spend the LAYER_16 quota. This is the phase that is actually supposed to raise high-layer MU pairing and DL cell capacity.</t>
         </is>
@@ -49189,25 +49157,25 @@
           <t>Children back to 0 first, master last.</t>
         </is>
       </c>
-      <c r="J9" s="268" t="inlineStr">
+      <c r="J9" s="267" t="inlineStr">
         <is>
           <t>PLANNED</t>
         </is>
       </c>
       <c r="K9" s="263" t="n"/>
     </row>
-    <row r="10" ht="75" customHeight="1">
-      <c r="A10" s="288" t="inlineStr">
+    <row r="10" ht="54.6" customHeight="1">
+      <c r="A10" s="287" t="inlineStr">
         <is>
           <t>Ph5</t>
         </is>
       </c>
-      <c r="B10" s="289" t="inlineStr">
+      <c r="B10" s="288" t="inlineStr">
         <is>
           <t>Ph4 + 7 days</t>
         </is>
       </c>
-      <c r="C10" s="290" t="inlineStr">
+      <c r="C10" s="289" t="inlineStr">
         <is>
           <t>Capacity upgrade layer: AHR Capacity Upgrade 2.0 and iBeam 2.0.</t>
         </is>
@@ -49234,25 +49202,25 @@
           <t>iBeam 2.0 children, then Phase2Sw=OFF, then the AHR CU bit.</t>
         </is>
       </c>
-      <c r="J10" s="268" t="inlineStr">
+      <c r="J10" s="267" t="inlineStr">
         <is>
           <t>PLANNED</t>
         </is>
       </c>
       <c r="K10" s="263" t="n"/>
     </row>
-    <row r="11" ht="75" customHeight="1">
-      <c r="A11" s="288" t="inlineStr">
+    <row r="11" ht="66" customHeight="1">
+      <c r="A11" s="287" t="inlineStr">
         <is>
           <t>Ph6</t>
         </is>
       </c>
-      <c r="B11" s="289" t="inlineStr">
+      <c r="B11" s="288" t="inlineStr">
         <is>
           <t>Ph5 + 7 days</t>
         </is>
       </c>
-      <c r="C11" s="290" t="inlineStr">
+      <c r="C11" s="289" t="inlineStr">
         <is>
           <t>UL side and the remaining weight variants.</t>
         </is>
@@ -49279,25 +49247,25 @@
           <t>One switch back per night, newest first.</t>
         </is>
       </c>
-      <c r="J11" s="268" t="inlineStr">
+      <c r="J11" s="267" t="inlineStr">
         <is>
           <t>PLANNED</t>
         </is>
       </c>
       <c r="K11" s="263" t="n"/>
     </row>
-    <row r="12" ht="75" customHeight="1">
-      <c r="A12" s="288" t="inlineStr">
+    <row r="12" ht="66" customHeight="1">
+      <c r="A12" s="287" t="inlineStr">
         <is>
           <t>Ph7</t>
         </is>
       </c>
-      <c r="B12" s="289" t="inlineStr">
+      <c r="B12" s="288" t="inlineStr">
         <is>
           <t>Ph6 + 14 days</t>
         </is>
       </c>
-      <c r="C12" s="290" t="inlineStr">
+      <c r="C12" s="289" t="inlineStr">
         <is>
           <t>Cluster rollout of the proven set.</t>
         </is>
@@ -49324,7 +49292,7 @@
           <t>Per-gNB rollback of that gNB's CME file only.</t>
         </is>
       </c>
-      <c r="J12" s="268" t="inlineStr">
+      <c r="J12" s="267" t="inlineStr">
         <is>
           <t>PLANNED</t>
         </is>
@@ -49333,7 +49301,7 @@
     </row>
     <row r="13" ht="8" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="291" t="inlineStr">
+      <c r="A14" s="290" t="inlineStr">
         <is>
           <t>Section 2.  Ph2 corrective sequence  —  the exact MML order that fixes the 10-Sep execution error</t>
         </is>
@@ -49423,8 +49391,8 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="67" customHeight="1">
-      <c r="A17" s="292" t="inlineStr">
+    <row r="17" ht="54.6" customHeight="1">
+      <c r="A17" s="291" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
@@ -49435,7 +49403,7 @@
 (alone)</t>
         </is>
       </c>
-      <c r="C17" s="293" t="inlineStr">
+      <c r="C17" s="292" t="inlineStr">
         <is>
           <t>MOD NRDUCELLSRS: NrDuCellId=102, SrsDetectionAlgoSwitch=SRS_IC_SW-0;</t>
         </is>
@@ -49469,18 +49437,18 @@
       </c>
       <c r="K17" s="263" t="n"/>
     </row>
-    <row r="18" ht="67" customHeight="1">
-      <c r="A18" s="292" t="inlineStr">
+    <row r="18" ht="54.6" customHeight="1">
+      <c r="A18" s="291" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="B18" s="294" t="inlineStr">
+      <c r="B18" s="293" t="inlineStr">
         <is>
           <t>Night 2</t>
         </is>
       </c>
-      <c r="C18" s="293" t="inlineStr">
+      <c r="C18" s="292" t="inlineStr">
         <is>
           <t>MOD NRDUCELLCHNCOVALGO: NrDuCellId=102, DlCoverageAlgoSwitch=SUPER_COVERAGE_SW-1;</t>
         </is>
@@ -49514,18 +49482,18 @@
       </c>
       <c r="K18" s="263" t="n"/>
     </row>
-    <row r="19" ht="67" customHeight="1">
-      <c r="A19" s="292" t="inlineStr">
+    <row r="19" ht="54.6" customHeight="1">
+      <c r="A19" s="291" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="B19" s="295" t="inlineStr">
+      <c r="B19" s="294" t="inlineStr">
         <is>
           <t>Night 2</t>
         </is>
       </c>
-      <c r="C19" s="293" t="inlineStr">
+      <c r="C19" s="292" t="inlineStr">
         <is>
           <t>MOD NRDUCELLBEAMALGO: NrDuCellId=102, WeightAlgoSwitch=SRS_WEIGHT_ESTIMATE_SW-1;</t>
         </is>
@@ -49559,18 +49527,18 @@
       </c>
       <c r="K19" s="263" t="n"/>
     </row>
-    <row r="20" ht="54" customHeight="1">
-      <c r="A20" s="292" t="inlineStr">
+    <row r="20" ht="43.2" customHeight="1">
+      <c r="A20" s="291" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="B20" s="294" t="inlineStr">
+      <c r="B20" s="293" t="inlineStr">
         <is>
           <t>Night 2</t>
         </is>
       </c>
-      <c r="C20" s="293" t="inlineStr">
+      <c r="C20" s="292" t="inlineStr">
         <is>
           <t>MOD NRDUCELLBEAMALGO: NrDuCellId=102, ChannelOptAlgoSwitch=BEAM_SELECT_OPT_SW-1;</t>
         </is>
@@ -49604,18 +49572,18 @@
       </c>
       <c r="K20" s="263" t="n"/>
     </row>
-    <row r="21" ht="67" customHeight="1">
-      <c r="A21" s="292" t="inlineStr">
+    <row r="21" ht="77.40000000000001" customHeight="1">
+      <c r="A21" s="291" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="B21" s="295" t="inlineStr">
+      <c r="B21" s="294" t="inlineStr">
         <is>
           <t>Night 2</t>
         </is>
       </c>
-      <c r="C21" s="293" t="inlineStr">
+      <c r="C21" s="292" t="inlineStr">
         <is>
           <t>MOD NRDUCELLBEAMALGO: NrDuCellId=102, BeamOptAlgoSwitch=BEAM_TRACKING_SW-1;</t>
         </is>
@@ -49649,18 +49617,18 @@
       </c>
       <c r="K21" s="263" t="n"/>
     </row>
-    <row r="22" ht="67" customHeight="1">
-      <c r="A22" s="292" t="inlineStr">
+    <row r="22" ht="54.6" customHeight="1">
+      <c r="A22" s="291" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="B22" s="294" t="inlineStr">
+      <c r="B22" s="293" t="inlineStr">
         <is>
           <t>Night 2</t>
         </is>
       </c>
-      <c r="C22" s="293" t="inlineStr">
+      <c r="C22" s="292" t="inlineStr">
         <is>
           <t>MOD NRDUCELLBEAMALGO: NrDuCellId=102, BeamOptAlgoSwitch=BEAM_TRACKING_SW-1&amp;INTELLIGENT_BEAM_SELECTION_SW-1;</t>
         </is>
@@ -49694,18 +49662,18 @@
       </c>
       <c r="K22" s="263" t="n"/>
     </row>
-    <row r="23" ht="67" customHeight="1">
-      <c r="A23" s="292" t="inlineStr">
+    <row r="23" ht="43.2" customHeight="1">
+      <c r="A23" s="291" t="inlineStr">
         <is>
           <t>2.7</t>
         </is>
       </c>
-      <c r="B23" s="295" t="inlineStr">
+      <c r="B23" s="294" t="inlineStr">
         <is>
           <t>Night 2</t>
         </is>
       </c>
-      <c r="C23" s="293" t="inlineStr">
+      <c r="C23" s="292" t="inlineStr">
         <is>
           <t>MOD NRDUCELLPDCCHALGO: NrDuCellId=102, AggLvlComprCceUsageThld=60;</t>
         </is>
@@ -49741,39 +49709,39 @@
     </row>
     <row r="24" ht="6" customHeight="1"/>
     <row r="25" ht="54" customHeight="1">
-      <c r="A25" s="296" t="inlineStr">
+      <c r="A25" s="295" t="inlineStr">
         <is>
           <t>Rollback for the whole of Ph2 night 2, in reverse order:  MOD NRDUCELLBEAMALGO BeamOptAlgoSwitch=BEAM_TRACKING_SW-0&amp;INTELLIGENT_BEAM_SELECTION_SW-0;  then ChannelOptAlgoSwitch=BEAM_SELECT_OPT_SW-0;  then WeightAlgoSwitch=SRS_WEIGHT_ESTIMATE_SW-0;  then MOD NRDUCELLCHNCOVALGO DlCoverageAlgoSwitch back to its pre-change value.  Do not touch HighPrecisionBeamSwitch, MaxMimoLayerNum, or the SU / MU / AHR Phase1 + Turbo bits.</t>
         </is>
       </c>
-      <c r="B25" s="276" t="n"/>
-      <c r="C25" s="276" t="n"/>
-      <c r="D25" s="276" t="n"/>
-      <c r="E25" s="276" t="n"/>
-      <c r="F25" s="276" t="n"/>
-      <c r="G25" s="276" t="n"/>
-      <c r="H25" s="276" t="n"/>
-      <c r="I25" s="276" t="n"/>
-      <c r="J25" s="276" t="n"/>
-      <c r="K25" s="276" t="n"/>
+      <c r="B25" s="275" t="n"/>
+      <c r="C25" s="275" t="n"/>
+      <c r="D25" s="275" t="n"/>
+      <c r="E25" s="275" t="n"/>
+      <c r="F25" s="275" t="n"/>
+      <c r="G25" s="275" t="n"/>
+      <c r="H25" s="275" t="n"/>
+      <c r="I25" s="275" t="n"/>
+      <c r="J25" s="275" t="n"/>
+      <c r="K25" s="275" t="n"/>
     </row>
     <row r="26" ht="8" customHeight="1"/>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="279" t="inlineStr">
+      <c r="A27" s="278" t="inlineStr">
         <is>
           <t>Section 3.  Ph3 to Ph7  —  switch list with its pre-requisite, in send order</t>
         </is>
       </c>
-      <c r="B27" s="280" t="n"/>
-      <c r="C27" s="280" t="n"/>
-      <c r="D27" s="280" t="n"/>
-      <c r="E27" s="280" t="n"/>
-      <c r="F27" s="280" t="n"/>
-      <c r="G27" s="280" t="n"/>
-      <c r="H27" s="280" t="n"/>
-      <c r="I27" s="280" t="n"/>
-      <c r="J27" s="280" t="n"/>
-      <c r="K27" s="280" t="n"/>
+      <c r="B27" s="279" t="n"/>
+      <c r="C27" s="279" t="n"/>
+      <c r="D27" s="279" t="n"/>
+      <c r="E27" s="279" t="n"/>
+      <c r="F27" s="279" t="n"/>
+      <c r="G27" s="279" t="n"/>
+      <c r="H27" s="279" t="n"/>
+      <c r="I27" s="279" t="n"/>
+      <c r="J27" s="279" t="n"/>
+      <c r="K27" s="279" t="n"/>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="16" t="inlineStr">
@@ -49793,74 +49761,74 @@
       <c r="K28" s="17" t="n"/>
     </row>
     <row r="29" ht="42" customHeight="1">
-      <c r="A29" s="281" t="inlineStr">
+      <c r="A29" s="280" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B29" s="281" t="inlineStr">
+      <c r="B29" s="280" t="inlineStr">
         <is>
           <t>Seq</t>
         </is>
       </c>
-      <c r="C29" s="281" t="inlineStr">
+      <c r="C29" s="280" t="inlineStr">
         <is>
           <t>Switch / parameter to enable</t>
         </is>
       </c>
-      <c r="D29" s="281" t="inlineStr">
+      <c r="D29" s="280" t="inlineStr">
         <is>
           <t>Pre-requisite switch / parameter  (must be ON first)</t>
         </is>
       </c>
-      <c r="E29" s="281" t="inlineStr">
+      <c r="E29" s="280" t="inlineStr">
         <is>
           <t>Pre-requisite MML  (run BEFORE this line)</t>
         </is>
       </c>
-      <c r="F29" s="281" t="inlineStr">
+      <c r="F29" s="280" t="inlineStr">
         <is>
           <t>Night</t>
         </is>
       </c>
-      <c r="G29" s="281" t="inlineStr">
+      <c r="G29" s="280" t="inlineStr">
         <is>
           <t>Counter to watch</t>
         </is>
       </c>
-      <c r="H29" s="281" t="inlineStr">
+      <c r="H29" s="280" t="inlineStr">
         <is>
           <t>Counter (continued)</t>
         </is>
       </c>
-      <c r="I29" s="281" t="inlineStr">
+      <c r="I29" s="280" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="J29" s="281" t="inlineStr">
+      <c r="J29" s="280" t="inlineStr">
         <is>
           <t>Note (continued)</t>
         </is>
       </c>
-      <c r="K29" s="281" t="inlineStr">
+      <c r="K29" s="280" t="inlineStr">
         <is>
           <t>Note (continued)</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="52" customHeight="1">
-      <c r="A30" s="297" t="inlineStr">
+    <row r="30" ht="43.2" customHeight="1">
+      <c r="A30" s="296" t="inlineStr">
         <is>
           <t>Ph3</t>
         </is>
       </c>
-      <c r="B30" s="295" t="inlineStr">
+      <c r="B30" s="294" t="inlineStr">
         <is>
           <t>Ph3.N1</t>
         </is>
       </c>
-      <c r="C30" s="293" t="inlineStr">
+      <c r="C30" s="292" t="inlineStr">
         <is>
           <t>DL_MU_PRECISE_SCH_SW-0</t>
         </is>
@@ -49875,7 +49843,7 @@
           <t>MOD NRDUCELLFEATURESW: NrDuCellId={NrDuCellId}, HighPrecisionBeamSwitch=ON;</t>
         </is>
       </c>
-      <c r="F30" s="295" t="inlineStr">
+      <c r="F30" s="294" t="inlineStr">
         <is>
           <t>N1</t>
         </is>
@@ -49894,18 +49862,18 @@
       <c r="J30" s="263" t="n"/>
       <c r="K30" s="263" t="n"/>
     </row>
-    <row r="31" ht="40" customHeight="1">
-      <c r="A31" s="297" t="inlineStr">
+    <row r="31" ht="43.2" customHeight="1">
+      <c r="A31" s="296" t="inlineStr">
         <is>
           <t>Ph3</t>
         </is>
       </c>
-      <c r="B31" s="294" t="inlineStr">
+      <c r="B31" s="293" t="inlineStr">
         <is>
           <t>Ph3.N2</t>
         </is>
       </c>
-      <c r="C31" s="293" t="inlineStr">
+      <c r="C31" s="292" t="inlineStr">
         <is>
           <t>DL_MU_ANTI_INTRF_SCH_SW-0</t>
         </is>
@@ -49920,7 +49888,7 @@
           <t>MOD NRDUCELLFEATURESW: NrDuCellId={NrDuCellId}, HighPrecisionBeamSwitch=ON;</t>
         </is>
       </c>
-      <c r="F31" s="294" t="inlineStr">
+      <c r="F31" s="293" t="inlineStr">
         <is>
           <t>N2</t>
         </is>
@@ -49939,18 +49907,18 @@
       <c r="J31" s="263" t="n"/>
       <c r="K31" s="263" t="n"/>
     </row>
-    <row r="32" ht="40" customHeight="1">
-      <c r="A32" s="297" t="inlineStr">
+    <row r="32" ht="43.2" customHeight="1">
+      <c r="A32" s="296" t="inlineStr">
         <is>
           <t>Ph3</t>
         </is>
       </c>
-      <c r="B32" s="295" t="inlineStr">
+      <c r="B32" s="294" t="inlineStr">
         <is>
           <t>Ph3.N3</t>
         </is>
       </c>
-      <c r="C32" s="293" t="inlineStr">
+      <c r="C32" s="292" t="inlineStr">
         <is>
           <t>SSB_BEAM_ADAPT_SW-1</t>
         </is>
@@ -49965,7 +49933,7 @@
           <t>LST NRDUCELLTRPBEAM: NrDuCellTrpId={NrDuCellTrpId};   // Tilt must not be 255</t>
         </is>
       </c>
-      <c r="F32" s="295" t="inlineStr">
+      <c r="F32" s="294" t="inlineStr">
         <is>
           <t>N3</t>
         </is>
@@ -49984,18 +49952,18 @@
       <c r="J32" s="263" t="n"/>
       <c r="K32" s="263" t="n"/>
     </row>
-    <row r="33" ht="40" customHeight="1">
-      <c r="A33" s="297" t="inlineStr">
+    <row r="33" ht="31.8" customHeight="1">
+      <c r="A33" s="296" t="inlineStr">
         <is>
           <t>Ph3</t>
         </is>
       </c>
-      <c r="B33" s="294" t="inlineStr">
+      <c r="B33" s="293" t="inlineStr">
         <is>
           <t>Ph3.N4</t>
         </is>
       </c>
-      <c r="C33" s="293" t="inlineStr">
+      <c r="C33" s="292" t="inlineStr">
         <is>
           <t>SSB_BEAM_VERTICAL_COV_IMP_SW-1</t>
         </is>
@@ -50010,7 +49978,7 @@
           <t>MOD NRDUCELLALGOSWITCH: NrDuCellId={NrDuCellId}, BeamOptSwitch=SSB_BEAM_ADAPT_SW-1;</t>
         </is>
       </c>
-      <c r="F33" s="294" t="inlineStr">
+      <c r="F33" s="293" t="inlineStr">
         <is>
           <t>N4</t>
         </is>
@@ -50029,18 +49997,18 @@
       <c r="J33" s="263" t="n"/>
       <c r="K33" s="263" t="n"/>
     </row>
-    <row r="34" ht="52" customHeight="1">
-      <c r="A34" s="297" t="inlineStr">
+    <row r="34" ht="43.2" customHeight="1">
+      <c r="A34" s="296" t="inlineStr">
         <is>
           <t>Ph4</t>
         </is>
       </c>
-      <c r="B34" s="295" t="inlineStr">
+      <c r="B34" s="294" t="inlineStr">
         <is>
           <t>Ph4.N1</t>
         </is>
       </c>
-      <c r="C34" s="293" t="inlineStr">
+      <c r="C34" s="292" t="inlineStr">
         <is>
           <t>HighLayerMuMimoSw=MMIMO_MULTILAYER_ENHANCE_SW-1</t>
         </is>
@@ -50055,7 +50023,7 @@
           <t>1) LST LICENSE;   2) LST NRDUCELLPDSCH: NrDuCellId={NrDuCellId};   // MaxMimoLayerNum</t>
         </is>
       </c>
-      <c r="F34" s="295" t="inlineStr">
+      <c r="F34" s="294" t="inlineStr">
         <is>
           <t>N1</t>
         </is>
@@ -50074,18 +50042,18 @@
       <c r="J34" s="263" t="n"/>
       <c r="K34" s="263" t="n"/>
     </row>
-    <row r="35" ht="40" customHeight="1">
-      <c r="A35" s="297" t="inlineStr">
+    <row r="35" ht="43.2" customHeight="1">
+      <c r="A35" s="296" t="inlineStr">
         <is>
           <t>Ph4</t>
         </is>
       </c>
-      <c r="B35" s="294" t="inlineStr">
+      <c r="B35" s="293" t="inlineStr">
         <is>
           <t>Ph4.N2</t>
         </is>
       </c>
-      <c r="C35" s="293" t="inlineStr">
+      <c r="C35" s="292" t="inlineStr">
         <is>
           <t>MU_RANK_BOOSTING_SW-1</t>
         </is>
@@ -50100,7 +50068,7 @@
           <t>MOD NRDUCELLDLMIMO: NrDuCellId={NrDuCellId}, HighLayerMuMimoSw=MMIMO_MULTILAYER_ENHANCE_SW-1;</t>
         </is>
       </c>
-      <c r="F35" s="294" t="inlineStr">
+      <c r="F35" s="293" t="inlineStr">
         <is>
           <t>N2</t>
         </is>
@@ -50119,18 +50087,18 @@
       <c r="J35" s="263" t="n"/>
       <c r="K35" s="263" t="n"/>
     </row>
-    <row r="36" ht="40" customHeight="1">
-      <c r="A36" s="297" t="inlineStr">
+    <row r="36" ht="43.2" customHeight="1">
+      <c r="A36" s="296" t="inlineStr">
         <is>
           <t>Ph4</t>
         </is>
       </c>
-      <c r="B36" s="295" t="inlineStr">
+      <c r="B36" s="294" t="inlineStr">
         <is>
           <t>Ph4.N3</t>
         </is>
       </c>
-      <c r="C36" s="293" t="inlineStr">
+      <c r="C36" s="292" t="inlineStr">
         <is>
           <t>MU_MIMO_PAIRING_PREFERRED_SW-1</t>
         </is>
@@ -50145,7 +50113,7 @@
           <t>MOD NRDUCELLDLMIMO: NrDuCellId={NrDuCellId}, HighLayerMuMimoSw=MMIMO_MULTILAYER_ENHANCE_SW-1;</t>
         </is>
       </c>
-      <c r="F36" s="295" t="inlineStr">
+      <c r="F36" s="294" t="inlineStr">
         <is>
           <t>N3</t>
         </is>
@@ -50164,18 +50132,18 @@
       <c r="J36" s="263" t="n"/>
       <c r="K36" s="263" t="n"/>
     </row>
-    <row r="37" ht="40" customHeight="1">
-      <c r="A37" s="297" t="inlineStr">
+    <row r="37" ht="43.2" customHeight="1">
+      <c r="A37" s="296" t="inlineStr">
         <is>
           <t>Ph4</t>
         </is>
       </c>
-      <c r="B37" s="294" t="inlineStr">
+      <c r="B37" s="293" t="inlineStr">
         <is>
           <t>Ph4.N4</t>
         </is>
       </c>
-      <c r="C37" s="293" t="inlineStr">
+      <c r="C37" s="292" t="inlineStr">
         <is>
           <t>SRS_MEAS_ACCELERATING_SW-1</t>
         </is>
@@ -50190,7 +50158,7 @@
           <t>MOD NRDUCELLDLMIMO: NrDuCellId={NrDuCellId}, HighLayerMuMimoSw=MMIMO_MULTILAYER_ENHANCE_SW-1;</t>
         </is>
       </c>
-      <c r="F37" s="294" t="inlineStr">
+      <c r="F37" s="293" t="inlineStr">
         <is>
           <t>N4</t>
         </is>
@@ -50209,18 +50177,18 @@
       <c r="J37" s="263" t="n"/>
       <c r="K37" s="263" t="n"/>
     </row>
-    <row r="38" ht="40" customHeight="1">
-      <c r="A38" s="297" t="inlineStr">
+    <row r="38" ht="31.8" customHeight="1">
+      <c r="A38" s="296" t="inlineStr">
         <is>
           <t>Ph5</t>
         </is>
       </c>
-      <c r="B38" s="295" t="inlineStr">
+      <c r="B38" s="294" t="inlineStr">
         <is>
           <t>Ph5.N1</t>
         </is>
       </c>
-      <c r="C38" s="293" t="inlineStr">
+      <c r="C38" s="292" t="inlineStr">
         <is>
           <t>AhrSwitch=AHR_CAPC_UPGRADE_PHASE2_SW-1</t>
         </is>
@@ -50235,7 +50203,7 @@
           <t>LST NRDUCELLFEATURESW: NrDuCellId={NrDuCellId};   // both AHR phases must be 1</t>
         </is>
       </c>
-      <c r="F38" s="295" t="inlineStr">
+      <c r="F38" s="294" t="inlineStr">
         <is>
           <t>N1</t>
         </is>
@@ -50254,18 +50222,18 @@
       <c r="J38" s="263" t="n"/>
       <c r="K38" s="263" t="n"/>
     </row>
-    <row r="39" ht="40" customHeight="1">
-      <c r="A39" s="297" t="inlineStr">
+    <row r="39" ht="43.2" customHeight="1">
+      <c r="A39" s="296" t="inlineStr">
         <is>
           <t>Ph5</t>
         </is>
       </c>
-      <c r="B39" s="294" t="inlineStr">
+      <c r="B39" s="293" t="inlineStr">
         <is>
           <t>Ph5.N2</t>
         </is>
       </c>
-      <c r="C39" s="293" t="inlineStr">
+      <c r="C39" s="292" t="inlineStr">
         <is>
           <t>PDCCH_MULTI_DIM_JOINT_SCH_SW-1</t>
         </is>
@@ -50280,7 +50248,7 @@
           <t>MOD NRDUCELLFEATURESW: NrDuCellId={NrDuCellId}, AhrSwitch=AHR_CAPC_UPGRADE_PHASE2_SW-1;</t>
         </is>
       </c>
-      <c r="F39" s="294" t="inlineStr">
+      <c r="F39" s="293" t="inlineStr">
         <is>
           <t>N2</t>
         </is>
@@ -50299,18 +50267,18 @@
       <c r="J39" s="263" t="n"/>
       <c r="K39" s="263" t="n"/>
     </row>
-    <row r="40" ht="52" customHeight="1">
-      <c r="A40" s="297" t="inlineStr">
+    <row r="40" ht="31.8" customHeight="1">
+      <c r="A40" s="296" t="inlineStr">
         <is>
           <t>Ph5</t>
         </is>
       </c>
-      <c r="B40" s="295" t="inlineStr">
+      <c r="B40" s="294" t="inlineStr">
         <is>
           <t>Ph5.N3</t>
         </is>
       </c>
-      <c r="C40" s="293" t="inlineStr">
+      <c r="C40" s="292" t="inlineStr">
         <is>
           <t>HighPrecisionBeamPhase2Sw=ON</t>
         </is>
@@ -50325,7 +50293,7 @@
           <t>MOD NRDUCELLFEATURESW: NrDuCellId={NrDuCellId}, HighPrecisionBeamSwitch=ON;</t>
         </is>
       </c>
-      <c r="F40" s="295" t="inlineStr">
+      <c r="F40" s="294" t="inlineStr">
         <is>
           <t>N3</t>
         </is>
@@ -50344,18 +50312,18 @@
       <c r="J40" s="263" t="n"/>
       <c r="K40" s="263" t="n"/>
     </row>
-    <row r="41" ht="40" customHeight="1">
-      <c r="A41" s="297" t="inlineStr">
+    <row r="41" ht="31.8" customHeight="1">
+      <c r="A41" s="296" t="inlineStr">
         <is>
           <t>Ph6</t>
         </is>
       </c>
-      <c r="B41" s="294" t="inlineStr">
+      <c r="B41" s="293" t="inlineStr">
         <is>
           <t>Ph6.N1</t>
         </is>
       </c>
-      <c r="C41" s="293" t="inlineStr">
+      <c r="C41" s="292" t="inlineStr">
         <is>
           <t>UL_LOW_NOISE_PHASE2_SW-1</t>
         </is>
@@ -50370,7 +50338,7 @@
           <t>1) DSP CLKTST;   2) LST NRDUCELLFEATURESW: NrDuCellId={NrDuCellId};</t>
         </is>
       </c>
-      <c r="F41" s="294" t="inlineStr">
+      <c r="F41" s="293" t="inlineStr">
         <is>
           <t>N1</t>
         </is>
@@ -50389,18 +50357,18 @@
       <c r="J41" s="263" t="n"/>
       <c r="K41" s="263" t="n"/>
     </row>
-    <row r="42" ht="40" customHeight="1">
-      <c r="A42" s="297" t="inlineStr">
+    <row r="42" ht="31.8" customHeight="1">
+      <c r="A42" s="296" t="inlineStr">
         <is>
           <t>Ph6</t>
         </is>
       </c>
-      <c r="B42" s="295" t="inlineStr">
+      <c r="B42" s="294" t="inlineStr">
         <is>
           <t>Ph6.N2</t>
         </is>
       </c>
-      <c r="C42" s="293" t="inlineStr">
+      <c r="C42" s="292" t="inlineStr">
         <is>
           <t>PUSCH_COORD_PWR_CTRL_SW-1</t>
         </is>
@@ -50415,7 +50383,7 @@
           <t>DSP CLKTST;   // must report time sync before coordinated PC</t>
         </is>
       </c>
-      <c r="F42" s="295" t="inlineStr">
+      <c r="F42" s="294" t="inlineStr">
         <is>
           <t>N2</t>
         </is>
@@ -50434,18 +50402,18 @@
       <c r="J42" s="263" t="n"/>
       <c r="K42" s="263" t="n"/>
     </row>
-    <row r="43" ht="52" customHeight="1">
-      <c r="A43" s="297" t="inlineStr">
+    <row r="43" ht="43.2" customHeight="1">
+      <c r="A43" s="296" t="inlineStr">
         <is>
           <t>Ph6</t>
         </is>
       </c>
-      <c r="B43" s="294" t="inlineStr">
+      <c r="B43" s="293" t="inlineStr">
         <is>
           <t>Ph6.N3</t>
         </is>
       </c>
-      <c r="C43" s="293" t="inlineStr">
+      <c r="C43" s="292" t="inlineStr">
         <is>
           <t>PMI_WEIGHT_OPT_SW-1</t>
         </is>
@@ -50460,7 +50428,7 @@
           <t>MOD NRDUCELLBEAMALGO: NrDuCellId={NrDuCellId}, BeamPerceiveMode=DISTRIBUTED_MODE;</t>
         </is>
       </c>
-      <c r="F43" s="294" t="inlineStr">
+      <c r="F43" s="293" t="inlineStr">
         <is>
           <t>N3</t>
         </is>
@@ -50479,18 +50447,18 @@
       <c r="J43" s="263" t="n"/>
       <c r="K43" s="263" t="n"/>
     </row>
-    <row r="44" ht="40" customHeight="1">
-      <c r="A44" s="297" t="inlineStr">
+    <row r="44" ht="31.8" customHeight="1">
+      <c r="A44" s="296" t="inlineStr">
         <is>
           <t>Ph7</t>
         </is>
       </c>
-      <c r="B44" s="295" t="inlineStr">
+      <c r="B44" s="294" t="inlineStr">
         <is>
           <t>Ph7.rolling</t>
         </is>
       </c>
-      <c r="C44" s="293" t="inlineStr">
+      <c r="C44" s="292" t="inlineStr">
         <is>
           <t>Green set from Ph2–Ph6, per gNB</t>
         </is>
@@ -50505,7 +50473,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="F44" s="295" t="inlineStr">
+      <c r="F44" s="294" t="inlineStr">
         <is>
           <t>rolling</t>
         </is>
@@ -50526,7 +50494,7 @@
     </row>
     <row r="45" ht="8" customHeight="1"/>
     <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="291" t="inlineStr">
+      <c r="A46" s="290" t="inlineStr">
         <is>
           <t>Section 4.  Execution rules for every phase from here on</t>
         </is>
@@ -50640,11 +50608,11 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="52" customHeight="1">
-      <c r="A51" s="272" t="n">
+    <row r="51" ht="43.2" customHeight="1">
+      <c r="A51" s="271" t="n">
         <v>1</v>
       </c>
-      <c r="B51" s="293" t="inlineStr">
+      <c r="B51" s="292" t="inlineStr">
         <is>
           <t>Pull N.SRS.NI.Avg, N.UL.SRS.PreSINR.Index*, DL IBLER, N.CCE.Used.Avg and N.PRB.DL.Used.Avg for 5–12 Sep, trial and neighbour control.</t>
         </is>
@@ -50657,29 +50625,29 @@
         </is>
       </c>
       <c r="F51" s="263" t="n"/>
-      <c r="G51" s="298" t="inlineStr">
+      <c r="G51" s="297" t="inlineStr">
         <is>
           <t>Performance</t>
         </is>
       </c>
-      <c r="H51" s="299" t="inlineStr">
+      <c r="H51" s="298" t="inlineStr">
         <is>
           <t>Ph2 work order is written</t>
         </is>
       </c>
       <c r="I51" s="263" t="n"/>
-      <c r="J51" s="300" t="inlineStr">
+      <c r="J51" s="299" t="inlineStr">
         <is>
           <t>Ph2</t>
         </is>
       </c>
       <c r="K51" s="263" t="n"/>
     </row>
-    <row r="52" ht="52" customHeight="1">
-      <c r="A52" s="274" t="n">
+    <row r="52" ht="31.8" customHeight="1">
+      <c r="A52" s="273" t="n">
         <v>2</v>
       </c>
-      <c r="B52" s="293" t="inlineStr">
+      <c r="B52" s="292" t="inlineStr">
         <is>
           <t>Run LST NRDUCELLCHNCOVALGO and LST NRDUCELLBEAMALGO on every trial cell (101 / 102 / 103 on each gNB).</t>
         </is>
@@ -50692,29 +50660,29 @@
         </is>
       </c>
       <c r="F52" s="263" t="n"/>
-      <c r="G52" s="298" t="inlineStr">
+      <c r="G52" s="297" t="inlineStr">
         <is>
           <t>O&amp;M</t>
         </is>
       </c>
-      <c r="H52" s="299" t="inlineStr">
+      <c r="H52" s="298" t="inlineStr">
         <is>
           <t>Ph2 night 2</t>
         </is>
       </c>
       <c r="I52" s="263" t="n"/>
-      <c r="J52" s="300" t="inlineStr">
+      <c r="J52" s="299" t="inlineStr">
         <is>
           <t>Ph2 steps 2.2–2.6</t>
         </is>
       </c>
       <c r="K52" s="263" t="n"/>
     </row>
-    <row r="53" ht="52" customHeight="1">
-      <c r="A53" s="272" t="n">
+    <row r="53" ht="31.8" customHeight="1">
+      <c r="A53" s="271" t="n">
         <v>3</v>
       </c>
-      <c r="B53" s="293" t="inlineStr">
+      <c r="B53" s="292" t="inlineStr">
         <is>
           <t>Re-issue the Ph2 work order as seven numbered single-switch MML lines with the pre-requisite column filled in from sheet 14.</t>
         </is>
@@ -50727,29 +50695,29 @@
         </is>
       </c>
       <c r="F53" s="263" t="n"/>
-      <c r="G53" s="298" t="inlineStr">
+      <c r="G53" s="297" t="inlineStr">
         <is>
           <t>RF / Optimisation</t>
         </is>
       </c>
-      <c r="H53" s="299" t="inlineStr">
+      <c r="H53" s="298" t="inlineStr">
         <is>
           <t>Next maintenance window</t>
         </is>
       </c>
       <c r="I53" s="263" t="n"/>
-      <c r="J53" s="300" t="inlineStr">
+      <c r="J53" s="299" t="inlineStr">
         <is>
           <t>Ph2</t>
         </is>
       </c>
       <c r="K53" s="263" t="n"/>
     </row>
-    <row r="54" ht="52" customHeight="1">
-      <c r="A54" s="274" t="n">
+    <row r="54" ht="31.8" customHeight="1">
+      <c r="A54" s="273" t="n">
         <v>4</v>
       </c>
-      <c r="B54" s="293" t="inlineStr">
+      <c r="B54" s="292" t="inlineStr">
         <is>
           <t>Retrieve the complete MML log with RETCODE for 10 and 11 Sep.</t>
         </is>
@@ -50762,29 +50730,29 @@
         </is>
       </c>
       <c r="F54" s="263" t="n"/>
-      <c r="G54" s="298" t="inlineStr">
+      <c r="G54" s="297" t="inlineStr">
         <is>
           <t>O&amp;M</t>
         </is>
       </c>
-      <c r="H54" s="299" t="inlineStr">
+      <c r="H54" s="298" t="inlineStr">
         <is>
           <t>Ph2 night 1</t>
         </is>
       </c>
       <c r="I54" s="263" t="n"/>
-      <c r="J54" s="300" t="inlineStr">
+      <c r="J54" s="299" t="inlineStr">
         <is>
           <t>Confidence in the whole Ph1 baseline</t>
         </is>
       </c>
       <c r="K54" s="263" t="n"/>
     </row>
-    <row r="55" ht="52" customHeight="1">
-      <c r="A55" s="272" t="n">
+    <row r="55" ht="31.8" customHeight="1">
+      <c r="A55" s="271" t="n">
         <v>5</v>
       </c>
-      <c r="B55" s="293" t="inlineStr">
+      <c r="B55" s="292" t="inlineStr">
         <is>
           <t>Confirm the DL user throughput figure in Mbit/s for 5, 9, 10, 11 and 12 Sep, trial and control.</t>
         </is>
@@ -50797,18 +50765,18 @@
         </is>
       </c>
       <c r="F55" s="263" t="n"/>
-      <c r="G55" s="298" t="inlineStr">
+      <c r="G55" s="297" t="inlineStr">
         <is>
           <t>Performance</t>
         </is>
       </c>
-      <c r="H55" s="299" t="inlineStr">
+      <c r="H55" s="298" t="inlineStr">
         <is>
           <t>Ph2 night 1</t>
         </is>
       </c>
       <c r="I55" s="263" t="n"/>
-      <c r="J55" s="300" t="inlineStr">
+      <c r="J55" s="299" t="inlineStr">
         <is>
           <t>Ph2 exit gate</t>
         </is>

</xml_diff>